<commit_message>
added gemma 4 results
</commit_message>
<xml_diff>
--- a/control/results/Control_Results.xlsx
+++ b/control/results/Control_Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\archlinux\home\omarg\VLMs-Medical-Imaging\control\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{505DC962-7451-4B2F-AA69-5C125EB7B042}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA04286E-C50D-476C-B808-24136B47E72F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{A77A01DF-2D44-4C38-8A9F-C029882A23C7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="31">
   <si>
     <t>Accuracy_Mean</t>
   </si>
@@ -127,6 +127,9 @@
   <si>
     <t>Qwen 3.5 9B (Thinking 2048)</t>
   </si>
+  <si>
+    <t>Gemma 4 27B A4B</t>
+  </si>
 </sst>
 </file>
 
@@ -156,7 +159,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -187,6 +190,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -201,7 +210,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -258,7 +267,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="1" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -282,6 +290,22 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="6" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="6" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -791,7 +815,7 @@
         <v>2</v>
       </c>
       <c r="R3" s="18">
-        <f t="shared" ref="R3:R28" si="0">AVERAGE(O3:Q3)/4878</f>
+        <f t="shared" ref="R3:R8" si="0">AVERAGE(O3:Q3)/4878</f>
         <v>1.3666803334700013E-4</v>
       </c>
     </row>
@@ -1226,16 +1250,16 @@
       <c r="B12" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="25">
+      <c r="C12" s="24">
         <v>0.50772174400000003</v>
       </c>
-      <c r="D12" s="25">
+      <c r="D12" s="24">
         <v>2.2488019999999998E-3</v>
       </c>
-      <c r="E12" s="25">
+      <c r="E12" s="24">
         <v>0.44327043300000002</v>
       </c>
-      <c r="F12" s="25">
+      <c r="F12" s="24">
         <v>3.465531E-3</v>
       </c>
       <c r="G12" s="20"/>
@@ -1279,16 +1303,16 @@
       <c r="B13" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="25">
+      <c r="C13" s="24">
         <v>0.91212245455787888</v>
       </c>
-      <c r="D13" s="25">
+      <c r="D13" s="24">
         <v>1.8601418052229669E-3</v>
       </c>
-      <c r="E13" s="25">
+      <c r="E13" s="24">
         <v>0.91224223361694312</v>
       </c>
-      <c r="F13" s="25">
+      <c r="F13" s="24">
         <v>1.8677504959338129E-3</v>
       </c>
       <c r="G13" s="20"/>
@@ -1332,16 +1356,16 @@
       <c r="B14" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C14" s="25">
+      <c r="C14" s="24">
         <v>0.8657919912532458</v>
       </c>
-      <c r="D14" s="25">
+      <c r="D14" s="24">
         <v>8.465699421046113E-3</v>
       </c>
-      <c r="E14" s="25">
+      <c r="E14" s="24">
         <v>0.86047402599161882</v>
       </c>
-      <c r="F14" s="25">
+      <c r="F14" s="24">
         <v>9.2095233660708202E-3</v>
       </c>
       <c r="G14" s="20"/>
@@ -1385,16 +1409,16 @@
       <c r="B15" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="25">
+      <c r="C15" s="24">
         <v>0.85137351400000005</v>
       </c>
-      <c r="D15" s="25">
+      <c r="D15" s="24">
         <v>8.8436469999999996E-3</v>
       </c>
-      <c r="E15" s="25">
+      <c r="E15" s="24">
         <v>0.84461146499999995</v>
       </c>
-      <c r="F15" s="25">
+      <c r="F15" s="24">
         <v>9.2031270000000002E-3</v>
       </c>
       <c r="G15" s="20"/>
@@ -1438,16 +1462,16 @@
       <c r="B16" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C16" s="25">
+      <c r="C16" s="24">
         <v>0.99788164548312153</v>
       </c>
-      <c r="D16" s="25">
+      <c r="D16" s="24">
         <v>3.1314580394668431E-4</v>
       </c>
-      <c r="E16" s="25">
+      <c r="E16" s="24">
         <v>0.99788008912124215</v>
       </c>
-      <c r="F16" s="25">
+      <c r="F16" s="24">
         <v>3.129263393627194E-4</v>
       </c>
       <c r="G16" s="20"/>
@@ -1491,16 +1515,16 @@
       <c r="B17" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C17" s="25">
+      <c r="C17" s="24">
         <v>0.99781331146644803</v>
       </c>
-      <c r="D17" s="25">
+      <c r="D17" s="24">
         <v>6.2629160789336863E-4</v>
       </c>
-      <c r="E17" s="25">
+      <c r="E17" s="24">
         <v>0.99780814404512586</v>
       </c>
-      <c r="F17" s="25">
+      <c r="F17" s="24">
         <v>6.2813094535919161E-4</v>
       </c>
       <c r="G17" s="20"/>
@@ -1544,16 +1568,16 @@
       <c r="B18" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C18" s="25">
+      <c r="C18" s="24">
         <v>0.99835998400000003</v>
       </c>
-      <c r="D18" s="25">
+      <c r="D18" s="24">
         <v>7.1014799999999996E-4</v>
       </c>
-      <c r="E18" s="25">
+      <c r="E18" s="24">
         <v>0.99835689599999999</v>
       </c>
-      <c r="F18" s="25">
+      <c r="F18" s="24">
         <v>7.1136300000000001E-4</v>
       </c>
       <c r="G18" s="20"/>
@@ -1597,16 +1621,16 @@
       <c r="B19" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C19" s="25">
+      <c r="C19" s="24">
         <v>0.99666666699999995</v>
       </c>
-      <c r="D19" s="25">
+      <c r="D19" s="24">
         <v>5.7735030000000001E-3</v>
       </c>
-      <c r="E19" s="25">
+      <c r="E19" s="24">
         <v>0.99616858200000002</v>
       </c>
-      <c r="F19" s="25">
+      <c r="F19" s="24">
         <v>6.63621E-3</v>
       </c>
       <c r="G19" s="20"/>
@@ -1650,16 +1674,16 @@
       <c r="B20" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C20" s="25">
+      <c r="C20" s="24">
         <v>0.98666666700000005</v>
       </c>
-      <c r="D20" s="25">
+      <c r="D20" s="24">
         <v>5.7735030000000001E-3</v>
       </c>
-      <c r="E20" s="25">
+      <c r="E20" s="24">
         <v>0.98458522699999995</v>
       </c>
-      <c r="F20" s="25">
+      <c r="F20" s="24">
         <v>6.7905400000000003E-3</v>
       </c>
       <c r="G20" s="20"/>
@@ -1703,16 +1727,16 @@
       <c r="B21" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C21" s="25">
+      <c r="C21" s="24">
         <v>0.99</v>
       </c>
-      <c r="D21" s="25">
+      <c r="D21" s="24">
         <v>0.01</v>
       </c>
-      <c r="E21" s="25">
+      <c r="E21" s="24">
         <v>0.98841664399999996</v>
       </c>
-      <c r="F21" s="25">
+      <c r="F21" s="24">
         <v>1.1628163E-2</v>
       </c>
       <c r="G21" s="20"/>
@@ -1756,49 +1780,49 @@
       <c r="B22" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="C22" s="23">
+      <c r="C22" s="22">
         <v>0.51400847341806744</v>
       </c>
-      <c r="D22" s="23">
+      <c r="D22" s="22">
         <v>5.1915866921477521E-3</v>
       </c>
-      <c r="E22" s="23">
+      <c r="E22" s="22">
         <v>0.49316103608265138</v>
       </c>
-      <c r="F22" s="23">
+      <c r="F22" s="22">
         <v>2.8052130075316619E-3</v>
       </c>
-      <c r="G22" s="24"/>
-      <c r="H22" s="24">
+      <c r="G22" s="23"/>
+      <c r="H22" s="23">
         <v>2498</v>
       </c>
-      <c r="I22" s="24">
+      <c r="I22" s="23">
         <v>2488</v>
       </c>
-      <c r="J22" s="24">
+      <c r="J22" s="23">
         <v>2536</v>
       </c>
-      <c r="K22" s="24">
+      <c r="K22" s="23">
         <v>2380</v>
       </c>
-      <c r="L22" s="24">
+      <c r="L22" s="23">
         <v>2390</v>
       </c>
-      <c r="M22" s="24">
+      <c r="M22" s="23">
         <v>2342</v>
       </c>
       <c r="N22" s="21"/>
-      <c r="O22" s="24">
+      <c r="O22" s="23">
         <v>178</v>
       </c>
-      <c r="P22" s="24">
+      <c r="P22" s="23">
         <v>157</v>
       </c>
-      <c r="Q22" s="24">
+      <c r="Q22" s="23">
         <v>163</v>
       </c>
       <c r="R22" s="19">
-        <f>AVERAGE(O22:Q22)/4878</f>
+        <f t="shared" ref="R22:R28" si="3">AVERAGE(O22:Q22)/4878</f>
         <v>3.4030340303403031E-2</v>
       </c>
     </row>
@@ -1809,49 +1833,49 @@
       <c r="B23" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="C23" s="23">
+      <c r="C23" s="22">
         <v>0.95223452234522343</v>
       </c>
-      <c r="D23" s="23">
+      <c r="D23" s="22">
         <v>2.1304437977476671E-3</v>
       </c>
-      <c r="E23" s="23">
+      <c r="E23" s="22">
         <v>0.95313001854960278</v>
       </c>
-      <c r="F23" s="23">
+      <c r="F23" s="22">
         <v>2.0237135866160239E-3</v>
       </c>
-      <c r="G23" s="24"/>
-      <c r="H23" s="24">
+      <c r="G23" s="23"/>
+      <c r="H23" s="23">
         <v>4633</v>
       </c>
-      <c r="I23" s="24">
+      <c r="I23" s="23">
         <v>4651</v>
       </c>
-      <c r="J23" s="24">
+      <c r="J23" s="23">
         <v>4651</v>
       </c>
-      <c r="K23" s="24">
+      <c r="K23" s="23">
         <v>245</v>
       </c>
-      <c r="L23" s="24">
+      <c r="L23" s="23">
         <v>227</v>
       </c>
-      <c r="M23" s="24">
+      <c r="M23" s="23">
         <v>227</v>
       </c>
       <c r="N23" s="21"/>
-      <c r="O23" s="24">
+      <c r="O23" s="23">
         <v>36</v>
       </c>
-      <c r="P23" s="24">
+      <c r="P23" s="23">
         <v>26</v>
       </c>
-      <c r="Q23" s="24">
+      <c r="Q23" s="23">
         <v>33</v>
       </c>
       <c r="R23" s="19">
-        <f>AVERAGE(O23:Q23)/4878</f>
+        <f t="shared" si="3"/>
         <v>6.491731583982507E-3</v>
       </c>
     </row>
@@ -1862,49 +1886,49 @@
       <c r="B24" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="C24" s="23">
+      <c r="C24" s="22">
         <v>0.92913762470958039</v>
       </c>
-      <c r="D24" s="23">
+      <c r="D24" s="22">
         <v>1.743522047584162E-3</v>
       </c>
-      <c r="E24" s="23">
+      <c r="E24" s="22">
         <v>0.9295337690884482</v>
       </c>
-      <c r="F24" s="23">
+      <c r="F24" s="22">
         <v>1.881165243078927E-3</v>
       </c>
-      <c r="G24" s="24"/>
-      <c r="H24" s="24">
+      <c r="G24" s="23"/>
+      <c r="H24" s="23">
         <v>4532</v>
       </c>
-      <c r="I24" s="24">
+      <c r="I24" s="23">
         <v>4524</v>
       </c>
-      <c r="J24" s="24">
+      <c r="J24" s="23">
         <v>4541</v>
       </c>
-      <c r="K24" s="24">
+      <c r="K24" s="23">
         <v>346</v>
       </c>
-      <c r="L24" s="24">
+      <c r="L24" s="23">
         <v>354</v>
       </c>
-      <c r="M24" s="24">
+      <c r="M24" s="23">
         <v>337</v>
       </c>
       <c r="N24" s="21"/>
-      <c r="O24" s="24">
+      <c r="O24" s="23">
         <v>34</v>
       </c>
-      <c r="P24" s="24">
+      <c r="P24" s="23">
         <v>44</v>
       </c>
-      <c r="Q24" s="24">
+      <c r="Q24" s="23">
         <v>56</v>
       </c>
       <c r="R24" s="19">
-        <f>AVERAGE(O24:Q24)/4878</f>
+        <f t="shared" si="3"/>
         <v>9.1567582342490083E-3</v>
       </c>
     </row>
@@ -1915,49 +1939,49 @@
       <c r="B25" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="C25" s="23">
+      <c r="C25" s="22">
         <v>0.92230422304223048</v>
       </c>
-      <c r="D25" s="23">
+      <c r="D25" s="22">
         <v>1.787166438516101E-3</v>
       </c>
-      <c r="E25" s="23">
+      <c r="E25" s="22">
         <v>0.92244431603482668</v>
       </c>
-      <c r="F25" s="23">
+      <c r="F25" s="22">
         <v>1.9619726873246158E-3</v>
       </c>
-      <c r="G25" s="24"/>
-      <c r="H25" s="24">
+      <c r="G25" s="23"/>
+      <c r="H25" s="23">
         <v>4505</v>
       </c>
-      <c r="I25" s="24">
+      <c r="I25" s="23">
         <v>4503</v>
       </c>
-      <c r="J25" s="24">
+      <c r="J25" s="23">
         <v>4489</v>
       </c>
-      <c r="K25" s="24">
+      <c r="K25" s="23">
         <v>373</v>
       </c>
-      <c r="L25" s="24">
+      <c r="L25" s="23">
         <v>375</v>
       </c>
-      <c r="M25" s="24">
+      <c r="M25" s="23">
         <v>389</v>
       </c>
       <c r="N25" s="21"/>
-      <c r="O25" s="24">
+      <c r="O25" s="23">
         <v>64</v>
       </c>
-      <c r="P25" s="24">
+      <c r="P25" s="23">
         <v>52</v>
       </c>
-      <c r="Q25" s="24">
+      <c r="Q25" s="23">
         <v>62</v>
       </c>
       <c r="R25" s="19">
-        <f>AVERAGE(O25:Q25)/4878</f>
+        <f t="shared" si="3"/>
         <v>1.2163454967883012E-2</v>
       </c>
     </row>
@@ -1968,49 +1992,49 @@
       <c r="B26" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="C26" s="23">
+      <c r="C26" s="22">
         <v>0.99794997949979503</v>
       </c>
-      <c r="D26" s="23">
+      <c r="D26" s="22">
         <v>3.5507396629127802E-4</v>
       </c>
-      <c r="E26" s="23">
+      <c r="E26" s="22">
         <v>0.99794779168915315</v>
       </c>
-      <c r="F26" s="23">
+      <c r="F26" s="22">
         <v>3.5492788432389232E-4</v>
       </c>
-      <c r="G26" s="24"/>
-      <c r="H26" s="24">
+      <c r="G26" s="23"/>
+      <c r="H26" s="23">
         <v>4869</v>
       </c>
-      <c r="I26" s="24">
+      <c r="I26" s="23">
         <v>4869</v>
       </c>
-      <c r="J26" s="24">
+      <c r="J26" s="23">
         <v>4866</v>
       </c>
-      <c r="K26" s="24">
+      <c r="K26" s="23">
         <v>9</v>
       </c>
-      <c r="L26" s="24">
+      <c r="L26" s="23">
         <v>9</v>
       </c>
-      <c r="M26" s="24">
+      <c r="M26" s="23">
         <v>12</v>
       </c>
       <c r="N26" s="21"/>
-      <c r="O26" s="24">
-        <v>0</v>
-      </c>
-      <c r="P26" s="24">
+      <c r="O26" s="23">
+        <v>0</v>
+      </c>
+      <c r="P26" s="23">
         <v>1</v>
       </c>
-      <c r="Q26" s="24">
+      <c r="Q26" s="23">
         <v>0</v>
       </c>
       <c r="R26" s="19">
-        <f>AVERAGE(O26:Q26)/4878</f>
+        <f t="shared" si="3"/>
         <v>6.8334016673500064E-5</v>
       </c>
     </row>
@@ -2021,49 +2045,49 @@
       <c r="B27" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="C27" s="23">
+      <c r="C27" s="22">
         <v>0.99822331556648902</v>
       </c>
-      <c r="D27" s="23">
+      <c r="D27" s="22">
         <v>5.1591051218194937E-4</v>
       </c>
-      <c r="E27" s="23">
+      <c r="E27" s="22">
         <v>0.9982200312317997</v>
       </c>
-      <c r="F27" s="23">
+      <c r="F27" s="22">
         <v>5.1641171693631114E-4</v>
       </c>
-      <c r="G27" s="24"/>
-      <c r="H27" s="24">
+      <c r="G27" s="23"/>
+      <c r="H27" s="23">
         <v>4869</v>
       </c>
-      <c r="I27" s="24">
+      <c r="I27" s="23">
         <v>4867</v>
       </c>
-      <c r="J27" s="24">
+      <c r="J27" s="23">
         <v>4872</v>
       </c>
-      <c r="K27" s="24">
+      <c r="K27" s="23">
         <v>9</v>
       </c>
-      <c r="L27" s="24">
+      <c r="L27" s="23">
         <v>11</v>
       </c>
-      <c r="M27" s="24">
+      <c r="M27" s="23">
         <v>6</v>
       </c>
       <c r="N27" s="21"/>
-      <c r="O27" s="24">
-        <v>0</v>
-      </c>
-      <c r="P27" s="24">
-        <v>0</v>
-      </c>
-      <c r="Q27" s="24">
+      <c r="O27" s="23">
+        <v>0</v>
+      </c>
+      <c r="P27" s="23">
+        <v>0</v>
+      </c>
+      <c r="Q27" s="23">
         <v>0</v>
       </c>
       <c r="R27" s="19">
-        <f>AVERAGE(O27:Q27)/4878</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -2074,49 +2098,49 @@
       <c r="B28" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="C28" s="23">
+      <c r="C28" s="22">
         <v>0.99842831761650952</v>
       </c>
-      <c r="D28" s="23">
+      <c r="D28" s="22">
         <v>6.5898939189509528E-4</v>
       </c>
-      <c r="E28" s="23">
+      <c r="E28" s="22">
         <v>0.99842566519779707</v>
       </c>
-      <c r="F28" s="23">
+      <c r="F28" s="22">
         <v>6.59459844255884E-4</v>
       </c>
-      <c r="G28" s="24"/>
-      <c r="H28" s="24">
+      <c r="G28" s="23"/>
+      <c r="H28" s="23">
         <v>4874</v>
       </c>
-      <c r="I28" s="24">
+      <c r="I28" s="23">
         <v>4869</v>
       </c>
-      <c r="J28" s="24">
+      <c r="J28" s="23">
         <v>4868</v>
       </c>
-      <c r="K28" s="24">
+      <c r="K28" s="23">
         <v>4</v>
       </c>
-      <c r="L28" s="24">
+      <c r="L28" s="23">
         <v>9</v>
       </c>
-      <c r="M28" s="24">
+      <c r="M28" s="23">
         <v>10</v>
       </c>
       <c r="N28" s="21"/>
-      <c r="O28" s="24">
-        <v>0</v>
-      </c>
-      <c r="P28" s="24">
+      <c r="O28" s="23">
+        <v>0</v>
+      </c>
+      <c r="P28" s="23">
         <v>1</v>
       </c>
-      <c r="Q28" s="24">
+      <c r="Q28" s="23">
         <v>0</v>
       </c>
       <c r="R28" s="19">
-        <f>AVERAGE(O28:Q28)/4878</f>
+        <f t="shared" si="3"/>
         <v>6.8334016673500064E-5</v>
       </c>
     </row>
@@ -2127,45 +2151,45 @@
       <c r="B29" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="C29" s="23">
+      <c r="C29" s="22">
         <v>1</v>
       </c>
-      <c r="D29" s="23">
-        <v>0</v>
-      </c>
-      <c r="E29" s="23">
+      <c r="D29" s="22">
+        <v>0</v>
+      </c>
+      <c r="E29" s="22">
         <v>1</v>
       </c>
-      <c r="F29" s="23">
-        <v>0</v>
-      </c>
-      <c r="G29" s="24"/>
-      <c r="H29" s="24">
+      <c r="F29" s="22">
+        <v>0</v>
+      </c>
+      <c r="G29" s="23"/>
+      <c r="H29" s="23">
         <v>100</v>
       </c>
-      <c r="I29" s="24">
+      <c r="I29" s="23">
         <v>100</v>
       </c>
-      <c r="J29" s="24">
+      <c r="J29" s="23">
         <v>100</v>
       </c>
-      <c r="K29" s="24">
-        <v>0</v>
-      </c>
-      <c r="L29" s="24">
-        <v>0</v>
-      </c>
-      <c r="M29" s="24">
+      <c r="K29" s="23">
+        <v>0</v>
+      </c>
+      <c r="L29" s="23">
+        <v>0</v>
+      </c>
+      <c r="M29" s="23">
         <v>0</v>
       </c>
       <c r="N29" s="21"/>
-      <c r="O29" s="24">
-        <v>0</v>
-      </c>
-      <c r="P29" s="24">
-        <v>0</v>
-      </c>
-      <c r="Q29" s="24">
+      <c r="O29" s="23">
+        <v>0</v>
+      </c>
+      <c r="P29" s="23">
+        <v>0</v>
+      </c>
+      <c r="Q29" s="23">
         <v>0</v>
       </c>
       <c r="R29" s="19">
@@ -2180,49 +2204,49 @@
       <c r="B30" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="C30" s="23">
+      <c r="C30" s="22">
         <v>0.99</v>
       </c>
-      <c r="D30" s="23">
-        <v>0</v>
-      </c>
-      <c r="E30" s="23">
+      <c r="D30" s="22">
+        <v>0</v>
+      </c>
+      <c r="E30" s="22">
         <v>0.9885057471264368</v>
       </c>
-      <c r="F30" s="23">
-        <v>0</v>
-      </c>
-      <c r="G30" s="24"/>
-      <c r="H30" s="24">
+      <c r="F30" s="22">
+        <v>0</v>
+      </c>
+      <c r="G30" s="23"/>
+      <c r="H30" s="23">
         <v>99</v>
       </c>
-      <c r="I30" s="24">
+      <c r="I30" s="23">
         <v>99</v>
       </c>
-      <c r="J30" s="24">
+      <c r="J30" s="23">
         <v>99</v>
       </c>
-      <c r="K30" s="24">
+      <c r="K30" s="23">
         <v>1</v>
       </c>
-      <c r="L30" s="24">
+      <c r="L30" s="23">
         <v>1</v>
       </c>
-      <c r="M30" s="24">
+      <c r="M30" s="23">
         <v>1</v>
       </c>
       <c r="N30" s="21"/>
-      <c r="O30" s="24">
-        <v>0</v>
-      </c>
-      <c r="P30" s="24">
-        <v>0</v>
-      </c>
-      <c r="Q30" s="24">
+      <c r="O30" s="23">
+        <v>0</v>
+      </c>
+      <c r="P30" s="23">
+        <v>0</v>
+      </c>
+      <c r="Q30" s="23">
         <v>0</v>
       </c>
       <c r="R30" s="19">
-        <f t="shared" ref="R30:R31" si="3">AVERAGE(O30:Q30)/100</f>
+        <f t="shared" ref="R30:R41" si="4">AVERAGE(O30:Q30)/100</f>
         <v>0</v>
       </c>
     </row>
@@ -2233,582 +2257,1109 @@
       <c r="B31" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="C31" s="23">
+      <c r="C31" s="22">
         <v>0.99333333333333329</v>
       </c>
-      <c r="D31" s="23">
+      <c r="D31" s="22">
         <v>5.7735026918962632E-3</v>
       </c>
-      <c r="E31" s="23">
+      <c r="E31" s="22">
         <v>0.9923371647509579</v>
       </c>
-      <c r="F31" s="23">
+      <c r="F31" s="22">
         <v>6.6362099906853459E-3</v>
       </c>
-      <c r="G31" s="24"/>
-      <c r="H31" s="24">
+      <c r="G31" s="23"/>
+      <c r="H31" s="23">
         <v>99</v>
       </c>
-      <c r="I31" s="24">
+      <c r="I31" s="23">
         <v>99</v>
       </c>
-      <c r="J31" s="24">
+      <c r="J31" s="23">
         <v>100</v>
       </c>
-      <c r="K31" s="24">
+      <c r="K31" s="23">
         <v>1</v>
       </c>
-      <c r="L31" s="24">
+      <c r="L31" s="23">
         <v>1</v>
       </c>
-      <c r="M31" s="24">
+      <c r="M31" s="23">
         <v>0</v>
       </c>
       <c r="N31" s="21"/>
-      <c r="O31" s="24">
-        <v>0</v>
-      </c>
-      <c r="P31" s="24">
-        <v>0</v>
-      </c>
-      <c r="Q31" s="24">
+      <c r="O31" s="23">
+        <v>0</v>
+      </c>
+      <c r="P31" s="23">
+        <v>0</v>
+      </c>
+      <c r="Q31" s="23">
         <v>0</v>
       </c>
       <c r="R31" s="19">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A32" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B32" s="32" t="s">
+        <v>21</v>
+      </c>
+      <c r="C32" s="33">
+        <v>0.50840508399999995</v>
+      </c>
+      <c r="D32" s="33">
+        <v>4.3196609999999998E-3</v>
+      </c>
+      <c r="E32" s="33">
+        <v>0.28273720299999999</v>
+      </c>
+      <c r="F32" s="33">
+        <v>7.8259000000000002E-3</v>
+      </c>
+      <c r="G32" s="32"/>
+      <c r="H32" s="32">
+        <v>2458</v>
+      </c>
+      <c r="I32" s="32">
+        <v>2500</v>
+      </c>
+      <c r="J32" s="32">
+        <v>2482</v>
+      </c>
+      <c r="K32" s="32">
+        <v>2420</v>
+      </c>
+      <c r="L32" s="32">
+        <v>2378</v>
+      </c>
+      <c r="M32" s="32">
+        <v>2396</v>
+      </c>
+      <c r="N32" s="34"/>
+      <c r="O32" s="32">
+        <v>0</v>
+      </c>
+      <c r="P32" s="32">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="32">
+        <v>0</v>
+      </c>
+      <c r="R32" s="35">
+        <f>AVERAGE(O32:Q32)/4878</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A33" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B33" s="36" t="s">
+        <v>18</v>
+      </c>
+      <c r="C33" s="33">
+        <v>0.5717507175071751</v>
+      </c>
+      <c r="D33" s="33">
+        <v>5.7070155420562256E-3</v>
+      </c>
+      <c r="E33" s="33">
+        <v>0.47200318217061771</v>
+      </c>
+      <c r="F33" s="33">
+        <v>1.167360688583105E-2</v>
+      </c>
+      <c r="G33" s="32"/>
+      <c r="H33" s="32">
+        <v>2764</v>
+      </c>
+      <c r="I33" s="32">
+        <v>2784</v>
+      </c>
+      <c r="J33" s="32">
+        <v>2819</v>
+      </c>
+      <c r="K33" s="32">
+        <v>2114</v>
+      </c>
+      <c r="L33" s="32">
+        <v>2094</v>
+      </c>
+      <c r="M33" s="32">
+        <v>2059</v>
+      </c>
+      <c r="N33" s="34"/>
+      <c r="O33" s="32">
+        <v>0</v>
+      </c>
+      <c r="P33" s="32">
+        <v>0</v>
+      </c>
+      <c r="Q33" s="32">
+        <v>0</v>
+      </c>
+      <c r="R33" s="35">
+        <f t="shared" ref="R33:R38" si="5">AVERAGE(O33:Q33)/4878</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A34" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B34" s="36" t="s">
+        <v>19</v>
+      </c>
+      <c r="C34" s="33">
+        <v>0.60386770499999998</v>
+      </c>
+      <c r="D34" s="33">
+        <v>6.738094E-3</v>
+      </c>
+      <c r="E34" s="33">
+        <v>0.55738297699999995</v>
+      </c>
+      <c r="F34" s="33">
+        <v>6.5843079999999997E-3</v>
+      </c>
+      <c r="G34" s="32"/>
+      <c r="H34" s="32">
+        <v>2982</v>
+      </c>
+      <c r="I34" s="32">
+        <v>2918</v>
+      </c>
+      <c r="J34" s="32">
+        <v>2937</v>
+      </c>
+      <c r="K34" s="32">
+        <v>1896</v>
+      </c>
+      <c r="L34" s="32">
+        <v>1960</v>
+      </c>
+      <c r="M34" s="32">
+        <v>1941</v>
+      </c>
+      <c r="N34" s="34"/>
+      <c r="O34" s="32">
+        <v>0</v>
+      </c>
+      <c r="P34" s="32">
+        <v>0</v>
+      </c>
+      <c r="Q34" s="32">
+        <v>0</v>
+      </c>
+      <c r="R34" s="35">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A35" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B35" s="36" t="s">
+        <v>20</v>
+      </c>
+      <c r="C35" s="33">
+        <v>0.578515785</v>
+      </c>
+      <c r="D35" s="33">
+        <v>4.0846370000000003E-3</v>
+      </c>
+      <c r="E35" s="33">
+        <v>0.49959096600000003</v>
+      </c>
+      <c r="F35" s="33">
+        <v>4.7357440000000001E-3</v>
+      </c>
+      <c r="G35" s="32"/>
+      <c r="H35" s="32">
+        <v>2834</v>
+      </c>
+      <c r="I35" s="32">
+        <v>2833</v>
+      </c>
+      <c r="J35" s="32">
+        <v>2799</v>
+      </c>
+      <c r="K35" s="32">
+        <v>2044</v>
+      </c>
+      <c r="L35" s="32">
+        <v>2045</v>
+      </c>
+      <c r="M35" s="32">
+        <v>2079</v>
+      </c>
+      <c r="N35" s="34"/>
+      <c r="O35" s="32">
+        <v>0</v>
+      </c>
+      <c r="P35" s="32">
+        <v>0</v>
+      </c>
+      <c r="Q35" s="32">
+        <v>0</v>
+      </c>
+      <c r="R35" s="35">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A36" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B36" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="C36" s="33">
+        <v>0.87337706699999995</v>
+      </c>
+      <c r="D36" s="33">
+        <v>7.9299850000000005E-3</v>
+      </c>
+      <c r="E36" s="33">
+        <v>0.87604022000000004</v>
+      </c>
+      <c r="F36" s="33">
+        <v>7.8775900000000003E-3</v>
+      </c>
+      <c r="G36" s="32"/>
+      <c r="H36" s="32">
+        <v>4301</v>
+      </c>
+      <c r="I36" s="32">
+        <v>4256</v>
+      </c>
+      <c r="J36" s="32">
+        <v>4224</v>
+      </c>
+      <c r="K36" s="32">
+        <v>577</v>
+      </c>
+      <c r="L36" s="32">
+        <v>622</v>
+      </c>
+      <c r="M36" s="32">
+        <v>654</v>
+      </c>
+      <c r="N36" s="34"/>
+      <c r="O36" s="32">
+        <v>0</v>
+      </c>
+      <c r="P36" s="32">
+        <v>0</v>
+      </c>
+      <c r="Q36" s="32">
+        <v>0</v>
+      </c>
+      <c r="R36" s="35">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A37" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B37" s="36" t="s">
+        <v>17</v>
+      </c>
+      <c r="C37" s="33">
+        <v>0.90105234400000001</v>
+      </c>
+      <c r="D37" s="33">
+        <v>9.24405E-4</v>
+      </c>
+      <c r="E37" s="33">
+        <v>0.90461120699999997</v>
+      </c>
+      <c r="F37" s="33">
+        <v>8.8342599999999998E-4</v>
+      </c>
+      <c r="G37" s="32"/>
+      <c r="H37" s="32">
+        <v>4400</v>
+      </c>
+      <c r="I37" s="32">
+        <v>4395</v>
+      </c>
+      <c r="J37" s="32">
+        <v>4391</v>
+      </c>
+      <c r="K37" s="32">
+        <v>478</v>
+      </c>
+      <c r="L37" s="32">
+        <v>483</v>
+      </c>
+      <c r="M37" s="32">
+        <v>487</v>
+      </c>
+      <c r="N37" s="34"/>
+      <c r="O37" s="32">
+        <v>0</v>
+      </c>
+      <c r="P37" s="32">
+        <v>0</v>
+      </c>
+      <c r="Q37" s="32">
+        <v>0</v>
+      </c>
+      <c r="R37" s="35">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A38" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B38" s="36" t="s">
+        <v>16</v>
+      </c>
+      <c r="C38" s="33">
+        <v>0.86176028400000004</v>
+      </c>
+      <c r="D38" s="33">
+        <v>4.921473E-3</v>
+      </c>
+      <c r="E38" s="33">
+        <v>0.86606366999999995</v>
+      </c>
+      <c r="F38" s="33">
+        <v>4.2672129999999997E-3</v>
+      </c>
+      <c r="G38" s="32"/>
+      <c r="H38" s="32">
+        <v>4228</v>
+      </c>
+      <c r="I38" s="32">
+        <v>4180</v>
+      </c>
+      <c r="J38" s="32">
+        <v>4203</v>
+      </c>
+      <c r="K38" s="32">
+        <v>650</v>
+      </c>
+      <c r="L38" s="32">
+        <v>698</v>
+      </c>
+      <c r="M38" s="32">
+        <v>675</v>
+      </c>
+      <c r="N38" s="34"/>
+      <c r="O38" s="32">
+        <v>0</v>
+      </c>
+      <c r="P38" s="32">
+        <v>0</v>
+      </c>
+      <c r="Q38" s="32">
+        <v>0</v>
+      </c>
+      <c r="R38" s="35">
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="B39" s="22"/>
+      <c r="A39" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B39" s="32" t="s">
+        <v>24</v>
+      </c>
+      <c r="C39" s="33">
+        <v>0.91</v>
+      </c>
+      <c r="D39" s="33">
+        <v>2.6457512999999998E-2</v>
+      </c>
+      <c r="E39" s="33">
+        <v>0.90546594999999996</v>
+      </c>
+      <c r="F39" s="33">
+        <v>2.6690629E-2</v>
+      </c>
+      <c r="G39" s="32"/>
+      <c r="H39" s="32">
+        <v>92</v>
+      </c>
+      <c r="I39" s="32">
+        <v>88</v>
+      </c>
+      <c r="J39" s="32">
+        <v>93</v>
+      </c>
+      <c r="K39" s="32">
+        <v>8</v>
+      </c>
+      <c r="L39" s="32">
+        <v>12</v>
+      </c>
+      <c r="M39" s="32">
+        <v>7</v>
+      </c>
+      <c r="N39" s="34"/>
+      <c r="O39" s="32">
+        <v>0</v>
+      </c>
+      <c r="P39" s="32">
+        <v>0</v>
+      </c>
+      <c r="Q39" s="32">
+        <v>0</v>
+      </c>
+      <c r="R39" s="35">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A40" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B40" s="32" t="s">
+        <v>23</v>
+      </c>
+      <c r="C40" s="33">
+        <v>0.943333333</v>
+      </c>
+      <c r="D40" s="33">
+        <v>1.5275252E-2</v>
+      </c>
+      <c r="E40" s="33">
+        <v>0.93624068400000005</v>
+      </c>
+      <c r="F40" s="33">
+        <v>1.75272E-2</v>
+      </c>
+      <c r="G40" s="32"/>
+      <c r="H40" s="32">
+        <v>94</v>
+      </c>
+      <c r="I40" s="32">
+        <v>96</v>
+      </c>
+      <c r="J40" s="32">
+        <v>93</v>
+      </c>
+      <c r="K40" s="32">
+        <v>6</v>
+      </c>
+      <c r="L40" s="32">
+        <v>4</v>
+      </c>
+      <c r="M40" s="32">
+        <v>7</v>
+      </c>
+      <c r="N40" s="34"/>
+      <c r="O40" s="32">
+        <v>0</v>
+      </c>
+      <c r="P40" s="32">
+        <v>0</v>
+      </c>
+      <c r="Q40" s="32">
+        <v>0</v>
+      </c>
+      <c r="R40" s="35">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A41" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B41" s="32" t="s">
+        <v>22</v>
+      </c>
+      <c r="C41" s="33">
+        <v>0.926666667</v>
+      </c>
+      <c r="D41" s="33">
+        <v>1.5275252E-2</v>
+      </c>
+      <c r="E41" s="33">
+        <v>0.91193344799999998</v>
+      </c>
+      <c r="F41" s="33">
+        <v>1.8782324999999999E-2</v>
+      </c>
+      <c r="G41" s="32"/>
+      <c r="H41" s="32">
+        <v>94</v>
+      </c>
+      <c r="I41" s="32">
+        <v>91</v>
+      </c>
+      <c r="J41" s="32">
+        <v>93</v>
+      </c>
+      <c r="K41" s="32">
+        <v>6</v>
+      </c>
+      <c r="L41" s="32">
+        <v>9</v>
+      </c>
+      <c r="M41" s="32">
+        <v>7</v>
+      </c>
+      <c r="N41" s="34"/>
+      <c r="O41" s="32">
+        <v>0</v>
+      </c>
+      <c r="P41" s="32">
+        <v>0</v>
+      </c>
+      <c r="Q41" s="32">
+        <v>0</v>
+      </c>
+      <c r="R41" s="35">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="42" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A42" s="26" t="s">
+      <c r="A42" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="B42" s="27" t="s">
+      <c r="B42" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="C42" s="28">
+      <c r="C42" s="27">
         <v>0.50505671723383894</v>
       </c>
-      <c r="D42" s="28">
+      <c r="D42" s="27">
         <v>6.6942926885477641E-3</v>
       </c>
-      <c r="E42" s="28">
+      <c r="E42" s="27">
         <v>0.4334698366828923</v>
       </c>
-      <c r="F42" s="28">
+      <c r="F42" s="27">
         <v>8.3271081394245688E-3</v>
       </c>
-      <c r="G42" s="28"/>
-      <c r="H42" s="27">
+      <c r="G42" s="27"/>
+      <c r="H42" s="26">
         <v>2484</v>
       </c>
-      <c r="I42" s="27">
+      <c r="I42" s="26">
         <v>2426</v>
       </c>
-      <c r="J42" s="27">
+      <c r="J42" s="26">
         <v>2481</v>
       </c>
-      <c r="K42" s="27">
+      <c r="K42" s="26">
         <v>2394</v>
       </c>
-      <c r="L42" s="27">
+      <c r="L42" s="26">
         <v>2452</v>
       </c>
-      <c r="M42" s="27">
+      <c r="M42" s="26">
         <v>2397</v>
       </c>
-      <c r="N42" s="29"/>
-      <c r="O42" s="27">
+      <c r="N42" s="28"/>
+      <c r="O42" s="26">
         <v>3</v>
       </c>
-      <c r="P42" s="27">
+      <c r="P42" s="26">
         <v>9</v>
       </c>
-      <c r="Q42" s="27">
+      <c r="Q42" s="26">
         <v>9</v>
       </c>
-      <c r="R42" s="30">
-        <f>AVERAGE(O42:Q42)/4878</f>
+      <c r="R42" s="29">
+        <f t="shared" ref="R42:R48" si="6">AVERAGE(O42:Q42)/4878</f>
         <v>1.4350143501435015E-3</v>
       </c>
     </row>
     <row r="43" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A43" s="26" t="s">
+      <c r="A43" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="B43" s="31" t="s">
+      <c r="B43" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="C43" s="28">
+      <c r="C43" s="27">
         <v>0.50061500615006149</v>
       </c>
-      <c r="D43" s="28">
+      <c r="D43" s="27">
         <v>7.3914540292413706E-4</v>
       </c>
-      <c r="E43" s="28">
+      <c r="E43" s="27">
         <v>0.60122211749517196</v>
       </c>
-      <c r="F43" s="28">
+      <c r="F43" s="27">
         <v>2.9606746648690071E-4</v>
       </c>
-      <c r="G43" s="28"/>
-      <c r="H43" s="27">
+      <c r="G43" s="27"/>
+      <c r="H43" s="26">
         <v>2445</v>
       </c>
-      <c r="I43" s="27">
+      <c r="I43" s="26">
         <v>2438</v>
       </c>
-      <c r="J43" s="27">
+      <c r="J43" s="26">
         <v>2443</v>
       </c>
-      <c r="K43" s="27">
+      <c r="K43" s="26">
         <v>2433</v>
       </c>
-      <c r="L43" s="27">
+      <c r="L43" s="26">
         <v>2440</v>
       </c>
-      <c r="M43" s="27">
+      <c r="M43" s="26">
         <v>2435</v>
       </c>
-      <c r="N43" s="29"/>
-      <c r="O43" s="27">
+      <c r="N43" s="28"/>
+      <c r="O43" s="26">
         <v>4</v>
       </c>
-      <c r="P43" s="27">
+      <c r="P43" s="26">
         <v>4</v>
       </c>
-      <c r="Q43" s="27">
+      <c r="Q43" s="26">
         <v>2</v>
       </c>
-      <c r="R43" s="30">
-        <f>AVERAGE(O43:Q43)/4878</f>
+      <c r="R43" s="29">
+        <f t="shared" si="6"/>
         <v>6.8334016673500075E-4</v>
       </c>
     </row>
     <row r="44" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A44" s="26" t="s">
+      <c r="A44" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="B44" s="31" t="s">
+      <c r="B44" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="C44" s="28">
+      <c r="C44" s="27">
         <v>0.50984009840098399</v>
       </c>
-      <c r="D44" s="28">
+      <c r="D44" s="27">
         <v>2.1695377704506399E-3</v>
       </c>
-      <c r="E44" s="28">
+      <c r="E44" s="27">
         <v>0.57842183136499792</v>
       </c>
-      <c r="F44" s="28">
+      <c r="F44" s="27">
         <v>2.8964055618430008E-3</v>
       </c>
-      <c r="G44" s="28"/>
-      <c r="H44" s="27">
+      <c r="G44" s="27"/>
+      <c r="H44" s="26">
         <v>2495</v>
       </c>
-      <c r="I44" s="27">
+      <c r="I44" s="26">
         <v>2475</v>
       </c>
-      <c r="J44" s="27">
+      <c r="J44" s="26">
         <v>2491</v>
       </c>
-      <c r="K44" s="27">
+      <c r="K44" s="26">
         <v>2383</v>
       </c>
-      <c r="L44" s="27">
+      <c r="L44" s="26">
         <v>2403</v>
       </c>
-      <c r="M44" s="27">
+      <c r="M44" s="26">
         <v>2387</v>
       </c>
-      <c r="N44" s="29"/>
-      <c r="O44" s="27">
+      <c r="N44" s="28"/>
+      <c r="O44" s="26">
         <v>3</v>
       </c>
-      <c r="P44" s="27">
+      <c r="P44" s="26">
         <v>6</v>
       </c>
-      <c r="Q44" s="27">
+      <c r="Q44" s="26">
         <v>2</v>
       </c>
-      <c r="R44" s="30">
-        <f>AVERAGE(O44:Q44)/4878</f>
+      <c r="R44" s="29">
+        <f t="shared" si="6"/>
         <v>7.5167418340850076E-4</v>
       </c>
     </row>
     <row r="45" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A45" s="26" t="s">
+      <c r="A45" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="B45" s="31" t="s">
+      <c r="B45" s="30" t="s">
         <v>20</v>
       </c>
-      <c r="C45" s="28">
+      <c r="C45" s="27">
         <v>0.50539838699999995</v>
       </c>
-      <c r="D45" s="28">
+      <c r="D45" s="27">
         <v>7.9193790000000007E-3</v>
       </c>
-      <c r="E45" s="28">
+      <c r="E45" s="27">
         <v>0.58867223300000004</v>
       </c>
-      <c r="F45" s="28">
+      <c r="F45" s="27">
         <v>4.3293189999999999E-3</v>
       </c>
-      <c r="G45" s="28"/>
-      <c r="H45" s="27">
+      <c r="G45" s="27"/>
+      <c r="H45" s="26">
         <v>2502</v>
       </c>
-      <c r="I45" s="27">
+      <c r="I45" s="26">
         <v>2425</v>
       </c>
-      <c r="J45" s="27">
+      <c r="J45" s="26">
         <v>2469</v>
       </c>
-      <c r="K45" s="27">
+      <c r="K45" s="26">
         <v>2376</v>
       </c>
-      <c r="L45" s="27">
+      <c r="L45" s="26">
         <v>2453</v>
       </c>
-      <c r="M45" s="27">
+      <c r="M45" s="26">
         <v>2409</v>
       </c>
-      <c r="N45" s="29"/>
-      <c r="O45" s="27">
+      <c r="N45" s="28"/>
+      <c r="O45" s="26">
         <v>6</v>
       </c>
-      <c r="P45" s="27">
+      <c r="P45" s="26">
         <v>5</v>
       </c>
-      <c r="Q45" s="27">
+      <c r="Q45" s="26">
         <v>2</v>
       </c>
-      <c r="R45" s="30">
-        <f>AVERAGE(O45:Q45)/4878</f>
+      <c r="R45" s="29">
+        <f t="shared" si="6"/>
         <v>8.8834221675550078E-4</v>
       </c>
     </row>
     <row r="46" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A46" s="26" t="s">
+      <c r="A46" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="B46" s="31" t="s">
+      <c r="B46" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C46" s="28">
+      <c r="C46" s="27">
         <v>0.540112068</v>
       </c>
-      <c r="D46" s="28">
+      <c r="D46" s="27">
         <v>6.8617019999999999E-3</v>
       </c>
-      <c r="E46" s="28">
+      <c r="E46" s="27">
         <v>0.60154494599999997</v>
       </c>
-      <c r="F46" s="28">
+      <c r="F46" s="27">
         <v>4.0854710000000002E-3</v>
       </c>
-      <c r="G46" s="28"/>
-      <c r="H46" s="27">
+      <c r="G46" s="27"/>
+      <c r="H46" s="26">
         <v>2661</v>
       </c>
-      <c r="I46" s="27">
+      <c r="I46" s="26">
         <v>2597</v>
       </c>
-      <c r="J46" s="27">
+      <c r="J46" s="26">
         <v>2646</v>
       </c>
-      <c r="K46" s="27">
+      <c r="K46" s="26">
         <v>2217</v>
       </c>
-      <c r="L46" s="27">
+      <c r="L46" s="26">
         <v>2281</v>
       </c>
-      <c r="M46" s="27">
+      <c r="M46" s="26">
         <v>2232</v>
       </c>
-      <c r="N46" s="29"/>
-      <c r="O46" s="27">
+      <c r="N46" s="28"/>
+      <c r="O46" s="26">
         <v>7</v>
       </c>
-      <c r="P46" s="27">
+      <c r="P46" s="26">
         <v>3</v>
       </c>
-      <c r="Q46" s="27">
+      <c r="Q46" s="26">
         <v>4</v>
       </c>
-      <c r="R46" s="30">
-        <f>AVERAGE(O46:Q46)/4878</f>
+      <c r="R46" s="29">
+        <f t="shared" si="6"/>
         <v>9.5667623342900101E-4</v>
       </c>
     </row>
     <row r="47" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A47" s="26" t="s">
+      <c r="A47" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="B47" s="31" t="s">
+      <c r="B47" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="C47" s="28">
+      <c r="C47" s="27">
         <v>0.50840508405084051</v>
       </c>
-      <c r="D47" s="28">
+      <c r="D47" s="27">
         <v>7.6347783720935357E-3</v>
       </c>
-      <c r="E47" s="28">
+      <c r="E47" s="27">
         <v>0.50859372912532019</v>
       </c>
-      <c r="F47" s="28">
+      <c r="F47" s="27">
         <v>8.6615013581022495E-3</v>
       </c>
-      <c r="G47" s="28"/>
-      <c r="H47" s="27">
+      <c r="G47" s="27"/>
+      <c r="H47" s="26">
         <v>2501</v>
       </c>
-      <c r="I47" s="27">
+      <c r="I47" s="26">
         <v>2502</v>
       </c>
-      <c r="J47" s="27">
+      <c r="J47" s="26">
         <v>2437</v>
       </c>
-      <c r="K47" s="27">
+      <c r="K47" s="26">
         <v>2377</v>
       </c>
-      <c r="L47" s="27">
+      <c r="L47" s="26">
         <v>2376</v>
       </c>
-      <c r="M47" s="27">
+      <c r="M47" s="26">
         <v>2441</v>
       </c>
-      <c r="N47" s="29"/>
-      <c r="O47" s="27">
+      <c r="N47" s="28"/>
+      <c r="O47" s="26">
         <v>12</v>
       </c>
-      <c r="P47" s="27">
+      <c r="P47" s="26">
         <v>6</v>
       </c>
-      <c r="Q47" s="27">
+      <c r="Q47" s="26">
         <v>6</v>
       </c>
-      <c r="R47" s="30">
-        <f>AVERAGE(O47:Q47)/4878</f>
+      <c r="R47" s="29">
+        <f t="shared" si="6"/>
         <v>1.6400164001640015E-3</v>
       </c>
     </row>
     <row r="48" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A48" s="26" t="s">
+      <c r="A48" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="B48" s="31" t="s">
+      <c r="B48" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="C48" s="28">
+      <c r="C48" s="27">
         <v>0.51359846899999995</v>
       </c>
-      <c r="D48" s="28">
+      <c r="D48" s="27">
         <v>5.7595479999999998E-3</v>
       </c>
-      <c r="E48" s="28">
+      <c r="E48" s="27">
         <v>0.37470842700000001</v>
       </c>
-      <c r="F48" s="28">
+      <c r="F48" s="27">
         <v>9.7275090000000005E-3</v>
       </c>
-      <c r="G48" s="28"/>
-      <c r="H48" s="27">
+      <c r="G48" s="27"/>
+      <c r="H48" s="26">
         <v>2508</v>
       </c>
-      <c r="I48" s="27">
+      <c r="I48" s="26">
         <v>2532</v>
       </c>
-      <c r="J48" s="27">
+      <c r="J48" s="26">
         <v>2476</v>
       </c>
-      <c r="K48" s="27">
+      <c r="K48" s="26">
         <v>2370</v>
       </c>
-      <c r="L48" s="27">
+      <c r="L48" s="26">
         <v>2346</v>
       </c>
-      <c r="M48" s="27">
+      <c r="M48" s="26">
         <v>2402</v>
       </c>
-      <c r="N48" s="29"/>
-      <c r="O48" s="27">
+      <c r="N48" s="28"/>
+      <c r="O48" s="26">
         <v>6</v>
       </c>
-      <c r="P48" s="27">
+      <c r="P48" s="26">
         <v>11</v>
       </c>
-      <c r="Q48" s="27">
+      <c r="Q48" s="26">
         <v>14</v>
       </c>
-      <c r="R48" s="30">
-        <f>AVERAGE(O48:Q48)/4878</f>
+      <c r="R48" s="29">
+        <f t="shared" si="6"/>
         <v>2.118354516878502E-3</v>
       </c>
     </row>
     <row r="49" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A49" s="26" t="s">
+      <c r="A49" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="B49" s="27" t="s">
+      <c r="B49" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="C49" s="28">
+      <c r="C49" s="27">
         <v>0.6</v>
       </c>
-      <c r="D49" s="28">
+      <c r="D49" s="27">
         <v>7.9372539331937678E-2</v>
       </c>
-      <c r="E49" s="28">
+      <c r="E49" s="27">
         <v>0.50077184316146961</v>
       </c>
-      <c r="F49" s="28">
+      <c r="F49" s="27">
         <v>9.2886313940835505E-2</v>
       </c>
-      <c r="G49" s="28"/>
-      <c r="H49" s="27">
+      <c r="G49" s="27"/>
+      <c r="H49" s="26">
         <v>57</v>
       </c>
-      <c r="I49" s="27">
+      <c r="I49" s="26">
         <v>69</v>
       </c>
-      <c r="J49" s="27">
+      <c r="J49" s="26">
         <v>54</v>
       </c>
-      <c r="K49" s="27">
+      <c r="K49" s="26">
         <v>43</v>
       </c>
-      <c r="L49" s="27">
+      <c r="L49" s="26">
         <v>31</v>
       </c>
-      <c r="M49" s="27">
+      <c r="M49" s="26">
         <v>46</v>
       </c>
-      <c r="N49" s="29"/>
-      <c r="O49" s="27">
-        <v>0</v>
-      </c>
-      <c r="P49" s="27">
-        <v>0</v>
-      </c>
-      <c r="Q49" s="27">
-        <v>0</v>
-      </c>
-      <c r="R49" s="30">
+      <c r="N49" s="28"/>
+      <c r="O49" s="26">
+        <v>0</v>
+      </c>
+      <c r="P49" s="26">
+        <v>0</v>
+      </c>
+      <c r="Q49" s="26">
+        <v>0</v>
+      </c>
+      <c r="R49" s="29">
         <f>AVERAGE(O49:Q49)/100</f>
         <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A50" s="26" t="s">
+      <c r="A50" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="B50" s="27" t="s">
+      <c r="B50" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="C50" s="28">
+      <c r="C50" s="27">
         <v>0.56000000000000005</v>
       </c>
-      <c r="D50" s="28">
+      <c r="D50" s="27">
         <v>4.3588989435406712E-2</v>
       </c>
-      <c r="E50" s="28">
+      <c r="E50" s="27">
         <v>0.37721511793123053</v>
       </c>
-      <c r="F50" s="28">
+      <c r="F50" s="27">
         <v>5.5728086685147657E-2</v>
       </c>
-      <c r="G50" s="28"/>
-      <c r="H50" s="27">
+      <c r="G50" s="27"/>
+      <c r="H50" s="26">
         <v>54</v>
       </c>
-      <c r="I50" s="27">
+      <c r="I50" s="26">
         <v>61</v>
       </c>
-      <c r="J50" s="27">
+      <c r="J50" s="26">
         <v>53</v>
       </c>
-      <c r="K50" s="27">
+      <c r="K50" s="26">
         <v>46</v>
       </c>
-      <c r="L50" s="27">
+      <c r="L50" s="26">
         <v>39</v>
       </c>
-      <c r="M50" s="27">
+      <c r="M50" s="26">
         <v>47</v>
       </c>
-      <c r="N50" s="29"/>
-      <c r="O50" s="27">
-        <v>0</v>
-      </c>
-      <c r="P50" s="27">
-        <v>0</v>
-      </c>
-      <c r="Q50" s="27">
+      <c r="N50" s="28"/>
+      <c r="O50" s="26">
+        <v>0</v>
+      </c>
+      <c r="P50" s="26">
+        <v>0</v>
+      </c>
+      <c r="Q50" s="26">
         <v>1</v>
       </c>
-      <c r="R50" s="30">
-        <f t="shared" ref="R50:R51" si="4">AVERAGE(O50:Q50)/100</f>
+      <c r="R50" s="29">
+        <f t="shared" ref="R50:R51" si="7">AVERAGE(O50:Q50)/100</f>
         <v>3.3333333333333331E-3</v>
       </c>
     </row>
     <row r="51" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A51" s="26" t="s">
+      <c r="A51" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="B51" s="27" t="s">
+      <c r="B51" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="C51" s="28">
+      <c r="C51" s="27">
         <v>0.54666666666666663</v>
       </c>
-      <c r="D51" s="28">
+      <c r="D51" s="27">
         <v>6.350852961085883E-2</v>
       </c>
-      <c r="E51" s="28">
+      <c r="E51" s="27">
         <v>0.19162624360364469</v>
       </c>
-      <c r="F51" s="28">
+      <c r="F51" s="27">
         <v>9.5545400524347388E-2</v>
       </c>
-      <c r="G51" s="28"/>
-      <c r="H51" s="27">
+      <c r="G51" s="27"/>
+      <c r="H51" s="26">
         <v>51</v>
       </c>
-      <c r="I51" s="27">
+      <c r="I51" s="26">
         <v>62</v>
       </c>
-      <c r="J51" s="27">
+      <c r="J51" s="26">
         <v>51</v>
       </c>
-      <c r="K51" s="27">
+      <c r="K51" s="26">
         <v>49</v>
       </c>
-      <c r="L51" s="27">
+      <c r="L51" s="26">
         <v>38</v>
       </c>
-      <c r="M51" s="27">
+      <c r="M51" s="26">
         <v>49</v>
       </c>
-      <c r="N51" s="29"/>
-      <c r="O51" s="27">
+      <c r="N51" s="28"/>
+      <c r="O51" s="26">
         <v>2</v>
       </c>
-      <c r="P51" s="27">
+      <c r="P51" s="26">
         <v>1</v>
       </c>
-      <c r="Q51" s="27">
+      <c r="Q51" s="26">
         <v>1</v>
       </c>
-      <c r="R51" s="30">
-        <f t="shared" si="4"/>
+      <c r="R51" s="29">
+        <f t="shared" si="7"/>
         <v>1.3333333333333332E-2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
commited gemma 4 4096 results
</commit_message>
<xml_diff>
--- a/control/results/Control_Results.xlsx
+++ b/control/results/Control_Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\archlinux\home\omarg\VLMs-Medical-Imaging\control\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA04286E-C50D-476C-B808-24136B47E72F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63040B22-617E-4B3C-B67C-5E5F3D3F1E4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{A77A01DF-2D44-4C38-8A9F-C029882A23C7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="33">
   <si>
     <t>Accuracy_Mean</t>
   </si>
@@ -130,6 +130,12 @@
   <si>
     <t>Gemma 4 27B A4B</t>
   </si>
+  <si>
+    <t>Gemma 4 27B A4B (4096)</t>
+  </si>
+  <si>
+    <t>Gemma 4 27B A4B (2048)</t>
+  </si>
 </sst>
 </file>
 
@@ -159,7 +165,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -192,7 +198,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79998168889431442"/>
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -210,7 +228,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -306,6 +324,35 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="7" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="7" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="8" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -643,7 +690,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD38333D-9F66-4DE8-9A2B-1755F063FACE}">
-  <dimension ref="A1:R51"/>
+  <dimension ref="A1:R71"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.6640625" customWidth="1"/>
@@ -2246,7 +2293,7 @@
         <v>0</v>
       </c>
       <c r="R30" s="19">
-        <f t="shared" ref="R30:R41" si="4">AVERAGE(O30:Q30)/100</f>
+        <f t="shared" ref="R30:R61" si="4">AVERAGE(O30:Q30)/100</f>
         <v>0</v>
       </c>
     </row>
@@ -2834,532 +2881,1332 @@
       </c>
     </row>
     <row r="42" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A42" s="25" t="s">
+      <c r="A42" s="43" t="s">
+        <v>32</v>
+      </c>
+      <c r="B42" s="44" t="s">
+        <v>21</v>
+      </c>
+      <c r="C42" s="45"/>
+      <c r="D42" s="45"/>
+      <c r="E42" s="45"/>
+      <c r="F42" s="45"/>
+      <c r="G42" s="45"/>
+      <c r="H42" s="45"/>
+      <c r="I42" s="45"/>
+      <c r="J42" s="45"/>
+      <c r="K42" s="45"/>
+      <c r="L42" s="45"/>
+      <c r="M42" s="45"/>
+      <c r="N42" s="45"/>
+      <c r="O42" s="45"/>
+      <c r="P42" s="45"/>
+      <c r="Q42" s="45"/>
+      <c r="R42" s="46" t="e">
+        <f>AVERAGE(O42:Q42)/4878</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="43" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A43" s="43" t="s">
+        <v>32</v>
+      </c>
+      <c r="B43" s="47" t="s">
+        <v>18</v>
+      </c>
+      <c r="C43" s="45"/>
+      <c r="D43" s="45"/>
+      <c r="E43" s="45"/>
+      <c r="F43" s="45"/>
+      <c r="G43" s="45"/>
+      <c r="H43" s="45"/>
+      <c r="I43" s="45"/>
+      <c r="J43" s="45"/>
+      <c r="K43" s="45"/>
+      <c r="L43" s="45"/>
+      <c r="M43" s="45"/>
+      <c r="N43" s="45"/>
+      <c r="O43" s="45"/>
+      <c r="P43" s="45"/>
+      <c r="Q43" s="45"/>
+      <c r="R43" s="46" t="e">
+        <f t="shared" ref="R43:R48" si="6">AVERAGE(O43:Q43)/4878</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="44" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A44" s="43" t="s">
+        <v>32</v>
+      </c>
+      <c r="B44" s="47" t="s">
+        <v>19</v>
+      </c>
+      <c r="C44" s="45"/>
+      <c r="D44" s="45"/>
+      <c r="E44" s="45"/>
+      <c r="F44" s="45"/>
+      <c r="G44" s="45"/>
+      <c r="H44" s="45"/>
+      <c r="I44" s="45"/>
+      <c r="J44" s="45"/>
+      <c r="K44" s="45"/>
+      <c r="L44" s="45"/>
+      <c r="M44" s="45"/>
+      <c r="N44" s="45"/>
+      <c r="O44" s="45"/>
+      <c r="P44" s="45"/>
+      <c r="Q44" s="45"/>
+      <c r="R44" s="46" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="45" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A45" s="43" t="s">
+        <v>32</v>
+      </c>
+      <c r="B45" s="47" t="s">
+        <v>20</v>
+      </c>
+      <c r="C45" s="45"/>
+      <c r="D45" s="45"/>
+      <c r="E45" s="45"/>
+      <c r="F45" s="45"/>
+      <c r="G45" s="45"/>
+      <c r="H45" s="45"/>
+      <c r="I45" s="45"/>
+      <c r="J45" s="45"/>
+      <c r="K45" s="45"/>
+      <c r="L45" s="45"/>
+      <c r="M45" s="45"/>
+      <c r="N45" s="45"/>
+      <c r="O45" s="45"/>
+      <c r="P45" s="45"/>
+      <c r="Q45" s="45"/>
+      <c r="R45" s="46" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="46" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A46" s="43" t="s">
+        <v>32</v>
+      </c>
+      <c r="B46" s="47" t="s">
+        <v>15</v>
+      </c>
+      <c r="C46" s="45"/>
+      <c r="D46" s="45"/>
+      <c r="E46" s="45"/>
+      <c r="F46" s="45"/>
+      <c r="G46" s="45"/>
+      <c r="H46" s="45"/>
+      <c r="I46" s="45"/>
+      <c r="J46" s="45"/>
+      <c r="K46" s="45"/>
+      <c r="L46" s="45"/>
+      <c r="M46" s="45"/>
+      <c r="N46" s="45"/>
+      <c r="O46" s="45"/>
+      <c r="P46" s="45"/>
+      <c r="Q46" s="45"/>
+      <c r="R46" s="46" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="47" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A47" s="43" t="s">
+        <v>32</v>
+      </c>
+      <c r="B47" s="47" t="s">
+        <v>17</v>
+      </c>
+      <c r="C47" s="45"/>
+      <c r="D47" s="45"/>
+      <c r="E47" s="45"/>
+      <c r="F47" s="45"/>
+      <c r="G47" s="45"/>
+      <c r="H47" s="45"/>
+      <c r="I47" s="45"/>
+      <c r="J47" s="45"/>
+      <c r="K47" s="45"/>
+      <c r="L47" s="45"/>
+      <c r="M47" s="45"/>
+      <c r="N47" s="45"/>
+      <c r="O47" s="45"/>
+      <c r="P47" s="45"/>
+      <c r="Q47" s="45"/>
+      <c r="R47" s="46" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="48" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A48" s="43" t="s">
+        <v>32</v>
+      </c>
+      <c r="B48" s="47" t="s">
+        <v>16</v>
+      </c>
+      <c r="C48" s="45"/>
+      <c r="D48" s="45"/>
+      <c r="E48" s="45"/>
+      <c r="F48" s="45"/>
+      <c r="G48" s="45"/>
+      <c r="H48" s="45"/>
+      <c r="I48" s="45"/>
+      <c r="J48" s="45"/>
+      <c r="K48" s="45"/>
+      <c r="L48" s="45"/>
+      <c r="M48" s="45"/>
+      <c r="N48" s="45"/>
+      <c r="O48" s="45"/>
+      <c r="P48" s="45"/>
+      <c r="Q48" s="45"/>
+      <c r="R48" s="46" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="49" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A49" s="43" t="s">
+        <v>32</v>
+      </c>
+      <c r="B49" s="44" t="s">
+        <v>24</v>
+      </c>
+      <c r="C49" s="45"/>
+      <c r="D49" s="45"/>
+      <c r="E49" s="45"/>
+      <c r="F49" s="45"/>
+      <c r="G49" s="45"/>
+      <c r="H49" s="45"/>
+      <c r="I49" s="45"/>
+      <c r="J49" s="45"/>
+      <c r="K49" s="45"/>
+      <c r="L49" s="45"/>
+      <c r="M49" s="45"/>
+      <c r="N49" s="45"/>
+      <c r="O49" s="45"/>
+      <c r="P49" s="45"/>
+      <c r="Q49" s="45"/>
+      <c r="R49" s="46" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="50" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A50" s="43" t="s">
+        <v>32</v>
+      </c>
+      <c r="B50" s="44" t="s">
+        <v>23</v>
+      </c>
+      <c r="C50" s="45"/>
+      <c r="D50" s="45"/>
+      <c r="E50" s="45"/>
+      <c r="F50" s="45"/>
+      <c r="G50" s="45"/>
+      <c r="H50" s="45"/>
+      <c r="I50" s="45"/>
+      <c r="J50" s="45"/>
+      <c r="K50" s="45"/>
+      <c r="L50" s="45"/>
+      <c r="M50" s="45"/>
+      <c r="N50" s="45"/>
+      <c r="O50" s="45"/>
+      <c r="P50" s="45"/>
+      <c r="Q50" s="45"/>
+      <c r="R50" s="46" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="51" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A51" s="43" t="s">
+        <v>32</v>
+      </c>
+      <c r="B51" s="44" t="s">
+        <v>22</v>
+      </c>
+      <c r="C51" s="45"/>
+      <c r="D51" s="45"/>
+      <c r="E51" s="45"/>
+      <c r="F51" s="45"/>
+      <c r="G51" s="45"/>
+      <c r="H51" s="45"/>
+      <c r="I51" s="45"/>
+      <c r="J51" s="45"/>
+      <c r="K51" s="45"/>
+      <c r="L51" s="45"/>
+      <c r="M51" s="45"/>
+      <c r="N51" s="45"/>
+      <c r="O51" s="45"/>
+      <c r="P51" s="45"/>
+      <c r="Q51" s="45"/>
+      <c r="R51" s="46" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="52" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A52" s="37" t="s">
+        <v>31</v>
+      </c>
+      <c r="B52" s="38" t="s">
+        <v>21</v>
+      </c>
+      <c r="C52" s="39">
+        <v>0.50560338900000001</v>
+      </c>
+      <c r="D52" s="39">
+        <v>4.0293899999999999E-3</v>
+      </c>
+      <c r="E52" s="39">
+        <v>0.485141023</v>
+      </c>
+      <c r="F52" s="39">
+        <v>6.7322099999999998E-3</v>
+      </c>
+      <c r="G52" s="38"/>
+      <c r="H52" s="38">
+        <v>2456</v>
+      </c>
+      <c r="I52" s="38">
+        <v>2454</v>
+      </c>
+      <c r="J52" s="38">
+        <v>2489</v>
+      </c>
+      <c r="K52" s="38">
+        <v>2422</v>
+      </c>
+      <c r="L52" s="38">
+        <v>2424</v>
+      </c>
+      <c r="M52" s="38">
+        <v>2389</v>
+      </c>
+      <c r="N52" s="40"/>
+      <c r="O52" s="38">
+        <v>41</v>
+      </c>
+      <c r="P52" s="38">
+        <v>37</v>
+      </c>
+      <c r="Q52" s="38">
+        <v>39</v>
+      </c>
+      <c r="R52" s="41">
+        <f>AVERAGE(O52:Q52)/4878</f>
+        <v>7.9950799507995073E-3</v>
+      </c>
+    </row>
+    <row r="53" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A53" s="37" t="s">
+        <v>31</v>
+      </c>
+      <c r="B53" s="42" t="s">
+        <v>18</v>
+      </c>
+      <c r="C53" s="39">
+        <v>0.93856771900000002</v>
+      </c>
+      <c r="D53" s="39">
+        <v>2.729942E-3</v>
+      </c>
+      <c r="E53" s="39">
+        <v>0.94105552299999995</v>
+      </c>
+      <c r="F53" s="39">
+        <v>2.5346430000000001E-3</v>
+      </c>
+      <c r="G53" s="38"/>
+      <c r="H53" s="38">
+        <v>4575</v>
+      </c>
+      <c r="I53" s="38">
+        <v>4593</v>
+      </c>
+      <c r="J53" s="38">
+        <v>4567</v>
+      </c>
+      <c r="K53" s="38">
+        <v>303</v>
+      </c>
+      <c r="L53" s="38">
+        <v>285</v>
+      </c>
+      <c r="M53" s="38">
+        <v>311</v>
+      </c>
+      <c r="N53" s="40"/>
+      <c r="O53" s="38">
+        <v>0</v>
+      </c>
+      <c r="P53" s="38">
+        <v>1</v>
+      </c>
+      <c r="Q53" s="38">
+        <v>1</v>
+      </c>
+      <c r="R53" s="41">
+        <f t="shared" ref="R53:R58" si="7">AVERAGE(O53:Q53)/4878</f>
+        <v>1.3666803334700013E-4</v>
+      </c>
+    </row>
+    <row r="54" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A54" s="37" t="s">
+        <v>31</v>
+      </c>
+      <c r="B54" s="42" t="s">
+        <v>19</v>
+      </c>
+      <c r="C54" s="39">
+        <v>0.88376383800000002</v>
+      </c>
+      <c r="D54" s="39">
+        <v>3.22186E-3</v>
+      </c>
+      <c r="E54" s="39">
+        <v>0.89130609599999999</v>
+      </c>
+      <c r="F54" s="39">
+        <v>2.8288850000000002E-3</v>
+      </c>
+      <c r="G54" s="38"/>
+      <c r="H54" s="38">
+        <v>4304</v>
+      </c>
+      <c r="I54" s="38">
+        <v>4329</v>
+      </c>
+      <c r="J54" s="38">
+        <v>4300</v>
+      </c>
+      <c r="K54" s="38">
+        <v>574</v>
+      </c>
+      <c r="L54" s="38">
+        <v>549</v>
+      </c>
+      <c r="M54" s="38">
+        <v>578</v>
+      </c>
+      <c r="N54" s="40"/>
+      <c r="O54" s="38">
+        <v>3</v>
+      </c>
+      <c r="P54" s="38">
+        <v>2</v>
+      </c>
+      <c r="Q54" s="38">
+        <v>3</v>
+      </c>
+      <c r="R54" s="41">
+        <f t="shared" si="7"/>
+        <v>5.4667213338800051E-4</v>
+      </c>
+    </row>
+    <row r="55" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A55" s="37" t="s">
+        <v>31</v>
+      </c>
+      <c r="B55" s="42" t="s">
+        <v>20</v>
+      </c>
+      <c r="C55" s="39">
+        <v>0.88711220400000002</v>
+      </c>
+      <c r="D55" s="39">
+        <v>6.2629199999999997E-4</v>
+      </c>
+      <c r="E55" s="39">
+        <v>0.89324033199999997</v>
+      </c>
+      <c r="F55" s="39">
+        <v>5.7067999999999995E-4</v>
+      </c>
+      <c r="G55" s="38"/>
+      <c r="H55" s="38">
+        <v>4330</v>
+      </c>
+      <c r="I55" s="38">
+        <v>4328</v>
+      </c>
+      <c r="J55" s="38">
+        <v>4324</v>
+      </c>
+      <c r="K55" s="38">
+        <v>548</v>
+      </c>
+      <c r="L55" s="38">
+        <v>550</v>
+      </c>
+      <c r="M55" s="38">
+        <v>554</v>
+      </c>
+      <c r="N55" s="40"/>
+      <c r="O55" s="38">
+        <v>3</v>
+      </c>
+      <c r="P55" s="38">
+        <v>2</v>
+      </c>
+      <c r="Q55" s="38">
+        <v>1</v>
+      </c>
+      <c r="R55" s="41">
+        <f t="shared" si="7"/>
+        <v>4.1000410004100039E-4</v>
+      </c>
+    </row>
+    <row r="56" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A56" s="37" t="s">
+        <v>31</v>
+      </c>
+      <c r="B56" s="42" t="s">
+        <v>15</v>
+      </c>
+      <c r="C56" s="39">
+        <v>0.99938499400000003</v>
+      </c>
+      <c r="D56" s="39">
+        <v>5.4238400000000003E-4</v>
+      </c>
+      <c r="E56" s="39">
+        <v>0.99938340699999995</v>
+      </c>
+      <c r="F56" s="39">
+        <v>5.4408899999999999E-4</v>
+      </c>
+      <c r="G56" s="38"/>
+      <c r="H56" s="38">
+        <v>4877</v>
+      </c>
+      <c r="I56" s="38">
+        <v>4872</v>
+      </c>
+      <c r="J56" s="38">
+        <v>4876</v>
+      </c>
+      <c r="K56" s="38">
+        <v>1</v>
+      </c>
+      <c r="L56" s="38">
+        <v>6</v>
+      </c>
+      <c r="M56" s="38">
+        <v>2</v>
+      </c>
+      <c r="N56" s="40"/>
+      <c r="O56" s="38">
+        <v>0</v>
+      </c>
+      <c r="P56" s="38">
+        <v>0</v>
+      </c>
+      <c r="Q56" s="38">
+        <v>0</v>
+      </c>
+      <c r="R56" s="41">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A57" s="37" t="s">
+        <v>31</v>
+      </c>
+      <c r="B57" s="42" t="s">
+        <v>17</v>
+      </c>
+      <c r="C57" s="39">
+        <v>0.99952166200000003</v>
+      </c>
+      <c r="D57" s="39">
+        <v>2.3671599999999999E-4</v>
+      </c>
+      <c r="E57" s="39">
+        <v>0.99952063700000005</v>
+      </c>
+      <c r="F57" s="39">
+        <v>2.3734799999999999E-4</v>
+      </c>
+      <c r="G57" s="38"/>
+      <c r="H57" s="38">
+        <v>4875</v>
+      </c>
+      <c r="I57" s="38">
+        <v>4875</v>
+      </c>
+      <c r="J57" s="38">
+        <v>4877</v>
+      </c>
+      <c r="K57" s="38">
+        <v>3</v>
+      </c>
+      <c r="L57" s="38">
+        <v>3</v>
+      </c>
+      <c r="M57" s="38">
+        <v>1</v>
+      </c>
+      <c r="N57" s="40"/>
+      <c r="O57" s="38">
+        <v>0</v>
+      </c>
+      <c r="P57" s="38">
+        <v>0</v>
+      </c>
+      <c r="Q57" s="38">
+        <v>0</v>
+      </c>
+      <c r="R57" s="41">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A58" s="37" t="s">
+        <v>31</v>
+      </c>
+      <c r="B58" s="42" t="s">
+        <v>16</v>
+      </c>
+      <c r="C58" s="39">
+        <v>1</v>
+      </c>
+      <c r="D58" s="39">
+        <v>0</v>
+      </c>
+      <c r="E58" s="39">
+        <v>1</v>
+      </c>
+      <c r="F58" s="39">
+        <v>0</v>
+      </c>
+      <c r="G58" s="38"/>
+      <c r="H58" s="38">
+        <v>4878</v>
+      </c>
+      <c r="I58" s="38">
+        <v>4878</v>
+      </c>
+      <c r="J58" s="38">
+        <v>4878</v>
+      </c>
+      <c r="K58" s="38">
+        <v>0</v>
+      </c>
+      <c r="L58" s="38">
+        <v>0</v>
+      </c>
+      <c r="M58" s="38">
+        <v>0</v>
+      </c>
+      <c r="N58" s="40"/>
+      <c r="O58" s="38">
+        <v>0</v>
+      </c>
+      <c r="P58" s="38">
+        <v>0</v>
+      </c>
+      <c r="Q58" s="38">
+        <v>0</v>
+      </c>
+      <c r="R58" s="41">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A59" s="37" t="s">
+        <v>31</v>
+      </c>
+      <c r="B59" s="38" t="s">
+        <v>24</v>
+      </c>
+      <c r="C59" s="39">
+        <v>1</v>
+      </c>
+      <c r="D59" s="39">
+        <v>0</v>
+      </c>
+      <c r="E59" s="39">
+        <v>1</v>
+      </c>
+      <c r="F59" s="39">
+        <v>0</v>
+      </c>
+      <c r="G59" s="38"/>
+      <c r="H59" s="38">
+        <v>100</v>
+      </c>
+      <c r="I59" s="38">
+        <v>100</v>
+      </c>
+      <c r="J59" s="38">
+        <v>100</v>
+      </c>
+      <c r="K59" s="38">
+        <v>0</v>
+      </c>
+      <c r="L59" s="38">
+        <v>0</v>
+      </c>
+      <c r="M59" s="38">
+        <v>0</v>
+      </c>
+      <c r="N59" s="40"/>
+      <c r="O59" s="38">
+        <v>0</v>
+      </c>
+      <c r="P59" s="38">
+        <v>0</v>
+      </c>
+      <c r="Q59" s="38">
+        <v>0</v>
+      </c>
+      <c r="R59" s="41">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A60" s="37" t="s">
+        <v>31</v>
+      </c>
+      <c r="B60" s="38" t="s">
+        <v>23</v>
+      </c>
+      <c r="C60" s="39">
+        <v>0.99666666699999995</v>
+      </c>
+      <c r="D60" s="39">
+        <v>5.7735030000000001E-3</v>
+      </c>
+      <c r="E60" s="39">
+        <v>0.99616858200000002</v>
+      </c>
+      <c r="F60" s="39">
+        <v>6.63621E-3</v>
+      </c>
+      <c r="G60" s="38"/>
+      <c r="H60" s="38">
+        <v>100</v>
+      </c>
+      <c r="I60" s="38">
+        <v>99</v>
+      </c>
+      <c r="J60" s="38">
+        <v>100</v>
+      </c>
+      <c r="K60" s="38">
+        <v>0</v>
+      </c>
+      <c r="L60" s="38">
+        <v>1</v>
+      </c>
+      <c r="M60" s="38">
+        <v>0</v>
+      </c>
+      <c r="N60" s="40"/>
+      <c r="O60" s="38">
+        <v>0</v>
+      </c>
+      <c r="P60" s="38">
+        <v>0</v>
+      </c>
+      <c r="Q60" s="38">
+        <v>0</v>
+      </c>
+      <c r="R60" s="41">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A61" s="37" t="s">
+        <v>31</v>
+      </c>
+      <c r="B61" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="C61" s="39">
+        <v>1</v>
+      </c>
+      <c r="D61" s="39">
+        <v>0</v>
+      </c>
+      <c r="E61" s="39">
+        <v>1</v>
+      </c>
+      <c r="F61" s="39">
+        <v>0</v>
+      </c>
+      <c r="G61" s="38"/>
+      <c r="H61" s="38">
+        <v>100</v>
+      </c>
+      <c r="I61" s="38">
+        <v>100</v>
+      </c>
+      <c r="J61" s="38">
+        <v>100</v>
+      </c>
+      <c r="K61" s="38">
+        <v>0</v>
+      </c>
+      <c r="L61" s="38">
+        <v>0</v>
+      </c>
+      <c r="M61" s="38">
+        <v>0</v>
+      </c>
+      <c r="N61" s="40"/>
+      <c r="O61" s="38">
+        <v>0</v>
+      </c>
+      <c r="P61" s="38">
+        <v>0</v>
+      </c>
+      <c r="Q61" s="38">
+        <v>0</v>
+      </c>
+      <c r="R61" s="41">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A62" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="B42" s="26" t="s">
+      <c r="B62" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="C42" s="27">
+      <c r="C62" s="27">
         <v>0.50505671723383894</v>
       </c>
-      <c r="D42" s="27">
+      <c r="D62" s="27">
         <v>6.6942926885477641E-3</v>
       </c>
-      <c r="E42" s="27">
+      <c r="E62" s="27">
         <v>0.4334698366828923</v>
       </c>
-      <c r="F42" s="27">
+      <c r="F62" s="27">
         <v>8.3271081394245688E-3</v>
       </c>
-      <c r="G42" s="27"/>
-      <c r="H42" s="26">
+      <c r="G62" s="27"/>
+      <c r="H62" s="26">
         <v>2484</v>
       </c>
-      <c r="I42" s="26">
+      <c r="I62" s="26">
         <v>2426</v>
       </c>
-      <c r="J42" s="26">
+      <c r="J62" s="26">
         <v>2481</v>
       </c>
-      <c r="K42" s="26">
+      <c r="K62" s="26">
         <v>2394</v>
       </c>
-      <c r="L42" s="26">
+      <c r="L62" s="26">
         <v>2452</v>
       </c>
-      <c r="M42" s="26">
+      <c r="M62" s="26">
         <v>2397</v>
       </c>
-      <c r="N42" s="28"/>
-      <c r="O42" s="26">
+      <c r="N62" s="28"/>
+      <c r="O62" s="26">
         <v>3</v>
       </c>
-      <c r="P42" s="26">
+      <c r="P62" s="26">
         <v>9</v>
       </c>
-      <c r="Q42" s="26">
+      <c r="Q62" s="26">
         <v>9</v>
       </c>
-      <c r="R42" s="29">
-        <f t="shared" ref="R42:R48" si="6">AVERAGE(O42:Q42)/4878</f>
+      <c r="R62" s="29">
+        <f t="shared" ref="R62:R68" si="8">AVERAGE(O62:Q62)/4878</f>
         <v>1.4350143501435015E-3</v>
       </c>
     </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A43" s="25" t="s">
+    <row r="63" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A63" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="B43" s="30" t="s">
+      <c r="B63" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="C43" s="27">
+      <c r="C63" s="27">
         <v>0.50061500615006149</v>
       </c>
-      <c r="D43" s="27">
+      <c r="D63" s="27">
         <v>7.3914540292413706E-4</v>
       </c>
-      <c r="E43" s="27">
+      <c r="E63" s="27">
         <v>0.60122211749517196</v>
       </c>
-      <c r="F43" s="27">
+      <c r="F63" s="27">
         <v>2.9606746648690071E-4</v>
       </c>
-      <c r="G43" s="27"/>
-      <c r="H43" s="26">
+      <c r="G63" s="27"/>
+      <c r="H63" s="26">
         <v>2445</v>
       </c>
-      <c r="I43" s="26">
+      <c r="I63" s="26">
         <v>2438</v>
       </c>
-      <c r="J43" s="26">
+      <c r="J63" s="26">
         <v>2443</v>
       </c>
-      <c r="K43" s="26">
+      <c r="K63" s="26">
         <v>2433</v>
       </c>
-      <c r="L43" s="26">
+      <c r="L63" s="26">
         <v>2440</v>
       </c>
-      <c r="M43" s="26">
+      <c r="M63" s="26">
         <v>2435</v>
       </c>
-      <c r="N43" s="28"/>
-      <c r="O43" s="26">
+      <c r="N63" s="28"/>
+      <c r="O63" s="26">
         <v>4</v>
       </c>
-      <c r="P43" s="26">
+      <c r="P63" s="26">
         <v>4</v>
       </c>
-      <c r="Q43" s="26">
+      <c r="Q63" s="26">
         <v>2</v>
       </c>
-      <c r="R43" s="29">
-        <f t="shared" si="6"/>
+      <c r="R63" s="29">
+        <f t="shared" si="8"/>
         <v>6.8334016673500075E-4</v>
       </c>
     </row>
-    <row r="44" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A44" s="25" t="s">
+    <row r="64" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A64" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="B44" s="30" t="s">
+      <c r="B64" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="C44" s="27">
+      <c r="C64" s="27">
         <v>0.50984009840098399</v>
       </c>
-      <c r="D44" s="27">
+      <c r="D64" s="27">
         <v>2.1695377704506399E-3</v>
       </c>
-      <c r="E44" s="27">
+      <c r="E64" s="27">
         <v>0.57842183136499792</v>
       </c>
-      <c r="F44" s="27">
+      <c r="F64" s="27">
         <v>2.8964055618430008E-3</v>
       </c>
-      <c r="G44" s="27"/>
-      <c r="H44" s="26">
+      <c r="G64" s="27"/>
+      <c r="H64" s="26">
         <v>2495</v>
       </c>
-      <c r="I44" s="26">
+      <c r="I64" s="26">
         <v>2475</v>
       </c>
-      <c r="J44" s="26">
+      <c r="J64" s="26">
         <v>2491</v>
       </c>
-      <c r="K44" s="26">
+      <c r="K64" s="26">
         <v>2383</v>
       </c>
-      <c r="L44" s="26">
+      <c r="L64" s="26">
         <v>2403</v>
       </c>
-      <c r="M44" s="26">
+      <c r="M64" s="26">
         <v>2387</v>
       </c>
-      <c r="N44" s="28"/>
-      <c r="O44" s="26">
+      <c r="N64" s="28"/>
+      <c r="O64" s="26">
         <v>3</v>
       </c>
-      <c r="P44" s="26">
+      <c r="P64" s="26">
         <v>6</v>
       </c>
-      <c r="Q44" s="26">
+      <c r="Q64" s="26">
         <v>2</v>
       </c>
-      <c r="R44" s="29">
-        <f t="shared" si="6"/>
+      <c r="R64" s="29">
+        <f t="shared" si="8"/>
         <v>7.5167418340850076E-4</v>
       </c>
     </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A45" s="25" t="s">
+    <row r="65" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A65" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="B45" s="30" t="s">
+      <c r="B65" s="30" t="s">
         <v>20</v>
       </c>
-      <c r="C45" s="27">
+      <c r="C65" s="27">
         <v>0.50539838699999995</v>
       </c>
-      <c r="D45" s="27">
+      <c r="D65" s="27">
         <v>7.9193790000000007E-3</v>
       </c>
-      <c r="E45" s="27">
+      <c r="E65" s="27">
         <v>0.58867223300000004</v>
       </c>
-      <c r="F45" s="27">
+      <c r="F65" s="27">
         <v>4.3293189999999999E-3</v>
       </c>
-      <c r="G45" s="27"/>
-      <c r="H45" s="26">
+      <c r="G65" s="27"/>
+      <c r="H65" s="26">
         <v>2502</v>
       </c>
-      <c r="I45" s="26">
+      <c r="I65" s="26">
         <v>2425</v>
       </c>
-      <c r="J45" s="26">
+      <c r="J65" s="26">
         <v>2469</v>
       </c>
-      <c r="K45" s="26">
+      <c r="K65" s="26">
         <v>2376</v>
       </c>
-      <c r="L45" s="26">
+      <c r="L65" s="26">
         <v>2453</v>
       </c>
-      <c r="M45" s="26">
+      <c r="M65" s="26">
         <v>2409</v>
       </c>
-      <c r="N45" s="28"/>
-      <c r="O45" s="26">
+      <c r="N65" s="28"/>
+      <c r="O65" s="26">
         <v>6</v>
       </c>
-      <c r="P45" s="26">
+      <c r="P65" s="26">
         <v>5</v>
       </c>
-      <c r="Q45" s="26">
+      <c r="Q65" s="26">
         <v>2</v>
       </c>
-      <c r="R45" s="29">
-        <f t="shared" si="6"/>
+      <c r="R65" s="29">
+        <f t="shared" si="8"/>
         <v>8.8834221675550078E-4</v>
       </c>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A46" s="25" t="s">
+    <row r="66" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A66" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="B46" s="30" t="s">
+      <c r="B66" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C46" s="27">
+      <c r="C66" s="27">
         <v>0.540112068</v>
       </c>
-      <c r="D46" s="27">
+      <c r="D66" s="27">
         <v>6.8617019999999999E-3</v>
       </c>
-      <c r="E46" s="27">
+      <c r="E66" s="27">
         <v>0.60154494599999997</v>
       </c>
-      <c r="F46" s="27">
+      <c r="F66" s="27">
         <v>4.0854710000000002E-3</v>
       </c>
-      <c r="G46" s="27"/>
-      <c r="H46" s="26">
+      <c r="G66" s="27"/>
+      <c r="H66" s="26">
         <v>2661</v>
       </c>
-      <c r="I46" s="26">
+      <c r="I66" s="26">
         <v>2597</v>
       </c>
-      <c r="J46" s="26">
+      <c r="J66" s="26">
         <v>2646</v>
       </c>
-      <c r="K46" s="26">
+      <c r="K66" s="26">
         <v>2217</v>
       </c>
-      <c r="L46" s="26">
+      <c r="L66" s="26">
         <v>2281</v>
       </c>
-      <c r="M46" s="26">
+      <c r="M66" s="26">
         <v>2232</v>
       </c>
-      <c r="N46" s="28"/>
-      <c r="O46" s="26">
+      <c r="N66" s="28"/>
+      <c r="O66" s="26">
         <v>7</v>
       </c>
-      <c r="P46" s="26">
+      <c r="P66" s="26">
         <v>3</v>
       </c>
-      <c r="Q46" s="26">
+      <c r="Q66" s="26">
         <v>4</v>
       </c>
-      <c r="R46" s="29">
-        <f t="shared" si="6"/>
+      <c r="R66" s="29">
+        <f t="shared" si="8"/>
         <v>9.5667623342900101E-4</v>
       </c>
     </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A47" s="25" t="s">
+    <row r="67" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A67" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="B47" s="30" t="s">
+      <c r="B67" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="C47" s="27">
+      <c r="C67" s="27">
         <v>0.50840508405084051</v>
       </c>
-      <c r="D47" s="27">
+      <c r="D67" s="27">
         <v>7.6347783720935357E-3</v>
       </c>
-      <c r="E47" s="27">
+      <c r="E67" s="27">
         <v>0.50859372912532019</v>
       </c>
-      <c r="F47" s="27">
+      <c r="F67" s="27">
         <v>8.6615013581022495E-3</v>
       </c>
-      <c r="G47" s="27"/>
-      <c r="H47" s="26">
+      <c r="G67" s="27"/>
+      <c r="H67" s="26">
         <v>2501</v>
       </c>
-      <c r="I47" s="26">
+      <c r="I67" s="26">
         <v>2502</v>
       </c>
-      <c r="J47" s="26">
+      <c r="J67" s="26">
         <v>2437</v>
       </c>
-      <c r="K47" s="26">
+      <c r="K67" s="26">
         <v>2377</v>
       </c>
-      <c r="L47" s="26">
+      <c r="L67" s="26">
         <v>2376</v>
       </c>
-      <c r="M47" s="26">
+      <c r="M67" s="26">
         <v>2441</v>
       </c>
-      <c r="N47" s="28"/>
-      <c r="O47" s="26">
+      <c r="N67" s="28"/>
+      <c r="O67" s="26">
         <v>12</v>
       </c>
-      <c r="P47" s="26">
+      <c r="P67" s="26">
         <v>6</v>
       </c>
-      <c r="Q47" s="26">
+      <c r="Q67" s="26">
         <v>6</v>
       </c>
-      <c r="R47" s="29">
-        <f t="shared" si="6"/>
+      <c r="R67" s="29">
+        <f t="shared" si="8"/>
         <v>1.6400164001640015E-3</v>
       </c>
     </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A48" s="25" t="s">
+    <row r="68" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A68" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="B48" s="30" t="s">
+      <c r="B68" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="C48" s="27">
+      <c r="C68" s="27">
         <v>0.51359846899999995</v>
       </c>
-      <c r="D48" s="27">
+      <c r="D68" s="27">
         <v>5.7595479999999998E-3</v>
       </c>
-      <c r="E48" s="27">
+      <c r="E68" s="27">
         <v>0.37470842700000001</v>
       </c>
-      <c r="F48" s="27">
+      <c r="F68" s="27">
         <v>9.7275090000000005E-3</v>
       </c>
-      <c r="G48" s="27"/>
-      <c r="H48" s="26">
+      <c r="G68" s="27"/>
+      <c r="H68" s="26">
         <v>2508</v>
       </c>
-      <c r="I48" s="26">
+      <c r="I68" s="26">
         <v>2532</v>
       </c>
-      <c r="J48" s="26">
+      <c r="J68" s="26">
         <v>2476</v>
       </c>
-      <c r="K48" s="26">
+      <c r="K68" s="26">
         <v>2370</v>
       </c>
-      <c r="L48" s="26">
+      <c r="L68" s="26">
         <v>2346</v>
       </c>
-      <c r="M48" s="26">
+      <c r="M68" s="26">
         <v>2402</v>
       </c>
-      <c r="N48" s="28"/>
-      <c r="O48" s="26">
+      <c r="N68" s="28"/>
+      <c r="O68" s="26">
         <v>6</v>
       </c>
-      <c r="P48" s="26">
+      <c r="P68" s="26">
         <v>11</v>
       </c>
-      <c r="Q48" s="26">
+      <c r="Q68" s="26">
         <v>14</v>
       </c>
-      <c r="R48" s="29">
-        <f t="shared" si="6"/>
+      <c r="R68" s="29">
+        <f t="shared" si="8"/>
         <v>2.118354516878502E-3</v>
       </c>
     </row>
-    <row r="49" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A49" s="25" t="s">
+    <row r="69" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A69" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="B49" s="26" t="s">
+      <c r="B69" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="C49" s="27">
+      <c r="C69" s="27">
         <v>0.6</v>
       </c>
-      <c r="D49" s="27">
+      <c r="D69" s="27">
         <v>7.9372539331937678E-2</v>
       </c>
-      <c r="E49" s="27">
+      <c r="E69" s="27">
         <v>0.50077184316146961</v>
       </c>
-      <c r="F49" s="27">
+      <c r="F69" s="27">
         <v>9.2886313940835505E-2</v>
       </c>
-      <c r="G49" s="27"/>
-      <c r="H49" s="26">
+      <c r="G69" s="27"/>
+      <c r="H69" s="26">
         <v>57</v>
       </c>
-      <c r="I49" s="26">
+      <c r="I69" s="26">
         <v>69</v>
       </c>
-      <c r="J49" s="26">
+      <c r="J69" s="26">
         <v>54</v>
       </c>
-      <c r="K49" s="26">
+      <c r="K69" s="26">
         <v>43</v>
       </c>
-      <c r="L49" s="26">
+      <c r="L69" s="26">
         <v>31</v>
       </c>
-      <c r="M49" s="26">
+      <c r="M69" s="26">
         <v>46</v>
       </c>
-      <c r="N49" s="28"/>
-      <c r="O49" s="26">
-        <v>0</v>
-      </c>
-      <c r="P49" s="26">
-        <v>0</v>
-      </c>
-      <c r="Q49" s="26">
-        <v>0</v>
-      </c>
-      <c r="R49" s="29">
-        <f>AVERAGE(O49:Q49)/100</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A50" s="25" t="s">
+      <c r="N69" s="28"/>
+      <c r="O69" s="26">
+        <v>0</v>
+      </c>
+      <c r="P69" s="26">
+        <v>0</v>
+      </c>
+      <c r="Q69" s="26">
+        <v>0</v>
+      </c>
+      <c r="R69" s="29">
+        <f>AVERAGE(O69:Q69)/100</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A70" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="B50" s="26" t="s">
+      <c r="B70" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="C50" s="27">
+      <c r="C70" s="27">
         <v>0.56000000000000005</v>
       </c>
-      <c r="D50" s="27">
+      <c r="D70" s="27">
         <v>4.3588989435406712E-2</v>
       </c>
-      <c r="E50" s="27">
+      <c r="E70" s="27">
         <v>0.37721511793123053</v>
       </c>
-      <c r="F50" s="27">
+      <c r="F70" s="27">
         <v>5.5728086685147657E-2</v>
       </c>
-      <c r="G50" s="27"/>
-      <c r="H50" s="26">
+      <c r="G70" s="27"/>
+      <c r="H70" s="26">
         <v>54</v>
       </c>
-      <c r="I50" s="26">
+      <c r="I70" s="26">
         <v>61</v>
       </c>
-      <c r="J50" s="26">
+      <c r="J70" s="26">
         <v>53</v>
       </c>
-      <c r="K50" s="26">
+      <c r="K70" s="26">
         <v>46</v>
       </c>
-      <c r="L50" s="26">
+      <c r="L70" s="26">
         <v>39</v>
       </c>
-      <c r="M50" s="26">
+      <c r="M70" s="26">
         <v>47</v>
       </c>
-      <c r="N50" s="28"/>
-      <c r="O50" s="26">
-        <v>0</v>
-      </c>
-      <c r="P50" s="26">
-        <v>0</v>
-      </c>
-      <c r="Q50" s="26">
+      <c r="N70" s="28"/>
+      <c r="O70" s="26">
+        <v>0</v>
+      </c>
+      <c r="P70" s="26">
+        <v>0</v>
+      </c>
+      <c r="Q70" s="26">
         <v>1</v>
       </c>
-      <c r="R50" s="29">
-        <f t="shared" ref="R50:R51" si="7">AVERAGE(O50:Q50)/100</f>
+      <c r="R70" s="29">
+        <f t="shared" ref="R70:R71" si="9">AVERAGE(O70:Q70)/100</f>
         <v>3.3333333333333331E-3</v>
       </c>
     </row>
-    <row r="51" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A51" s="25" t="s">
+    <row r="71" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A71" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="B51" s="26" t="s">
+      <c r="B71" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="C51" s="27">
+      <c r="C71" s="27">
         <v>0.54666666666666663</v>
       </c>
-      <c r="D51" s="27">
+      <c r="D71" s="27">
         <v>6.350852961085883E-2</v>
       </c>
-      <c r="E51" s="27">
+      <c r="E71" s="27">
         <v>0.19162624360364469</v>
       </c>
-      <c r="F51" s="27">
+      <c r="F71" s="27">
         <v>9.5545400524347388E-2</v>
       </c>
-      <c r="G51" s="27"/>
-      <c r="H51" s="26">
+      <c r="G71" s="27"/>
+      <c r="H71" s="26">
         <v>51</v>
       </c>
-      <c r="I51" s="26">
+      <c r="I71" s="26">
         <v>62</v>
       </c>
-      <c r="J51" s="26">
+      <c r="J71" s="26">
         <v>51</v>
       </c>
-      <c r="K51" s="26">
+      <c r="K71" s="26">
         <v>49</v>
       </c>
-      <c r="L51" s="26">
+      <c r="L71" s="26">
         <v>38</v>
       </c>
-      <c r="M51" s="26">
+      <c r="M71" s="26">
         <v>49</v>
       </c>
-      <c r="N51" s="28"/>
-      <c r="O51" s="26">
+      <c r="N71" s="28"/>
+      <c r="O71" s="26">
         <v>2</v>
       </c>
-      <c r="P51" s="26">
+      <c r="P71" s="26">
         <v>1</v>
       </c>
-      <c r="Q51" s="26">
+      <c r="Q71" s="26">
         <v>1</v>
       </c>
-      <c r="R51" s="29">
-        <f t="shared" si="7"/>
+      <c r="R71" s="29">
+        <f t="shared" si="9"/>
         <v>1.3333333333333332E-2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added gemma 4 2048
</commit_message>
<xml_diff>
--- a/control/results/Control_Results.xlsx
+++ b/control/results/Control_Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\archlinux\home\omarg\VLMs-Medical-Imaging\control\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63040B22-617E-4B3C-B67C-5E5F3D3F1E4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F613AACF-2F38-41C4-808B-EC912457FF7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{A77A01DF-2D44-4C38-8A9F-C029882A23C7}"/>
   </bookViews>
@@ -228,7 +228,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -354,6 +354,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="8" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -707,6 +710,7 @@
     <col min="15" max="15" width="13.109375" customWidth="1"/>
     <col min="16" max="16" width="12.6640625" customWidth="1"/>
     <col min="17" max="17" width="14.5546875" customWidth="1"/>
+    <col min="18" max="18" width="13.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.3">
@@ -2887,24 +2891,50 @@
       <c r="B42" s="44" t="s">
         <v>21</v>
       </c>
-      <c r="C42" s="45"/>
-      <c r="D42" s="45"/>
-      <c r="E42" s="45"/>
-      <c r="F42" s="45"/>
+      <c r="C42" s="48">
+        <v>0.491731584</v>
+      </c>
+      <c r="D42" s="48">
+        <v>4.0293899999999999E-3</v>
+      </c>
+      <c r="E42" s="48">
+        <v>0.47180090800000002</v>
+      </c>
+      <c r="F42" s="48">
+        <v>5.2481669999999998E-3</v>
+      </c>
       <c r="G42" s="45"/>
-      <c r="H42" s="45"/>
-      <c r="I42" s="45"/>
-      <c r="J42" s="45"/>
-      <c r="K42" s="45"/>
-      <c r="L42" s="45"/>
-      <c r="M42" s="45"/>
+      <c r="H42" s="44">
+        <v>2384</v>
+      </c>
+      <c r="I42" s="44">
+        <v>2391</v>
+      </c>
+      <c r="J42" s="44">
+        <v>2421</v>
+      </c>
+      <c r="K42" s="44">
+        <v>2494</v>
+      </c>
+      <c r="L42" s="44">
+        <v>2487</v>
+      </c>
+      <c r="M42" s="44">
+        <v>2457</v>
+      </c>
       <c r="N42" s="45"/>
-      <c r="O42" s="45"/>
-      <c r="P42" s="45"/>
-      <c r="Q42" s="45"/>
-      <c r="R42" s="46" t="e">
+      <c r="O42" s="44">
+        <v>167</v>
+      </c>
+      <c r="P42" s="44">
+        <v>192</v>
+      </c>
+      <c r="Q42" s="44">
+        <v>165</v>
+      </c>
+      <c r="R42" s="46">
         <f>AVERAGE(O42:Q42)/4878</f>
-        <v>#DIV/0!</v>
+        <v>3.5807024736914037E-2</v>
       </c>
     </row>
     <row r="43" spans="1:18" x14ac:dyDescent="0.3">
@@ -2914,24 +2944,50 @@
       <c r="B43" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="C43" s="45"/>
-      <c r="D43" s="45"/>
-      <c r="E43" s="45"/>
-      <c r="F43" s="45"/>
+      <c r="C43" s="48">
+        <v>0.93966106299999996</v>
+      </c>
+      <c r="D43" s="48">
+        <v>2.0120860000000002E-3</v>
+      </c>
+      <c r="E43" s="48">
+        <v>0.94197917600000003</v>
+      </c>
+      <c r="F43" s="48">
+        <v>1.9816259999999998E-3</v>
+      </c>
       <c r="G43" s="45"/>
-      <c r="H43" s="45"/>
-      <c r="I43" s="45"/>
-      <c r="J43" s="45"/>
-      <c r="K43" s="45"/>
-      <c r="L43" s="45"/>
-      <c r="M43" s="45"/>
+      <c r="H43" s="44">
+        <v>4595</v>
+      </c>
+      <c r="I43" s="44">
+        <v>4578</v>
+      </c>
+      <c r="J43" s="44">
+        <v>4578</v>
+      </c>
+      <c r="K43" s="44">
+        <v>283</v>
+      </c>
+      <c r="L43" s="44">
+        <v>300</v>
+      </c>
+      <c r="M43" s="44">
+        <v>300</v>
+      </c>
       <c r="N43" s="45"/>
-      <c r="O43" s="45"/>
-      <c r="P43" s="45"/>
-      <c r="Q43" s="45"/>
-      <c r="R43" s="46" t="e">
+      <c r="O43" s="44">
+        <v>13</v>
+      </c>
+      <c r="P43" s="44">
+        <v>27</v>
+      </c>
+      <c r="Q43" s="44">
+        <v>11</v>
+      </c>
+      <c r="R43" s="46">
         <f t="shared" ref="R43:R48" si="6">AVERAGE(O43:Q43)/4878</f>
-        <v>#DIV/0!</v>
+        <v>3.4850348503485036E-3</v>
       </c>
     </row>
     <row r="44" spans="1:18" x14ac:dyDescent="0.3">
@@ -2941,24 +2997,50 @@
       <c r="B44" s="47" t="s">
         <v>19</v>
       </c>
-      <c r="C44" s="45"/>
-      <c r="D44" s="45"/>
-      <c r="E44" s="45"/>
-      <c r="F44" s="45"/>
+      <c r="C44" s="48">
+        <v>0.88068880699999996</v>
+      </c>
+      <c r="D44" s="48">
+        <v>4.6431950000000001E-3</v>
+      </c>
+      <c r="E44" s="48">
+        <v>0.88809610400000005</v>
+      </c>
+      <c r="F44" s="48">
+        <v>4.1396489999999996E-3</v>
+      </c>
       <c r="G44" s="45"/>
-      <c r="H44" s="45"/>
-      <c r="I44" s="45"/>
-      <c r="J44" s="45"/>
-      <c r="K44" s="45"/>
-      <c r="L44" s="45"/>
-      <c r="M44" s="45"/>
+      <c r="H44" s="44">
+        <v>4272</v>
+      </c>
+      <c r="I44" s="44">
+        <v>4299</v>
+      </c>
+      <c r="J44" s="44">
+        <v>4317</v>
+      </c>
+      <c r="K44" s="44">
+        <v>606</v>
+      </c>
+      <c r="L44" s="44">
+        <v>579</v>
+      </c>
+      <c r="M44" s="44">
+        <v>561</v>
+      </c>
       <c r="N44" s="45"/>
-      <c r="O44" s="45"/>
-      <c r="P44" s="45"/>
-      <c r="Q44" s="45"/>
-      <c r="R44" s="46" t="e">
+      <c r="O44" s="44">
+        <v>44</v>
+      </c>
+      <c r="P44" s="44">
+        <v>43</v>
+      </c>
+      <c r="Q44" s="44">
+        <v>39</v>
+      </c>
+      <c r="R44" s="46">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
+        <v>8.6100861008610082E-3</v>
       </c>
     </row>
     <row r="45" spans="1:18" x14ac:dyDescent="0.3">
@@ -2968,24 +3050,50 @@
       <c r="B45" s="47" t="s">
         <v>20</v>
       </c>
-      <c r="C45" s="45"/>
-      <c r="D45" s="45"/>
-      <c r="E45" s="45"/>
-      <c r="F45" s="45"/>
+      <c r="C45" s="48">
+        <v>0.878502118</v>
+      </c>
+      <c r="D45" s="48">
+        <v>2.7067520000000002E-3</v>
+      </c>
+      <c r="E45" s="48">
+        <v>0.88537760899999995</v>
+      </c>
+      <c r="F45" s="48">
+        <v>2.6429919999999998E-3</v>
+      </c>
       <c r="G45" s="45"/>
-      <c r="H45" s="45"/>
-      <c r="I45" s="45"/>
-      <c r="J45" s="45"/>
-      <c r="K45" s="45"/>
-      <c r="L45" s="45"/>
-      <c r="M45" s="45"/>
+      <c r="H45" s="44">
+        <v>4288</v>
+      </c>
+      <c r="I45" s="44">
+        <v>4271</v>
+      </c>
+      <c r="J45" s="44">
+        <v>4297</v>
+      </c>
+      <c r="K45" s="44">
+        <v>590</v>
+      </c>
+      <c r="L45" s="44">
+        <v>607</v>
+      </c>
+      <c r="M45" s="44">
+        <v>581</v>
+      </c>
       <c r="N45" s="45"/>
-      <c r="O45" s="45"/>
-      <c r="P45" s="45"/>
-      <c r="Q45" s="45"/>
-      <c r="R45" s="46" t="e">
+      <c r="O45" s="44">
+        <v>45</v>
+      </c>
+      <c r="P45" s="44">
+        <v>54</v>
+      </c>
+      <c r="Q45" s="44">
+        <v>37</v>
+      </c>
+      <c r="R45" s="46">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
+        <v>9.2934262675960101E-3</v>
       </c>
     </row>
     <row r="46" spans="1:18" x14ac:dyDescent="0.3">
@@ -2995,24 +3103,50 @@
       <c r="B46" s="47" t="s">
         <v>15</v>
       </c>
-      <c r="C46" s="45"/>
-      <c r="D46" s="45"/>
-      <c r="E46" s="45"/>
-      <c r="F46" s="45"/>
+      <c r="C46" s="48">
+        <v>0.99911165800000001</v>
+      </c>
+      <c r="D46" s="48">
+        <v>5.1591099999999997E-4</v>
+      </c>
+      <c r="E46" s="48">
+        <v>0.99910933999999996</v>
+      </c>
+      <c r="F46" s="48">
+        <v>5.1775400000000004E-4</v>
+      </c>
       <c r="G46" s="45"/>
-      <c r="H46" s="45"/>
-      <c r="I46" s="45"/>
-      <c r="J46" s="45"/>
-      <c r="K46" s="45"/>
-      <c r="L46" s="45"/>
-      <c r="M46" s="45"/>
+      <c r="H46" s="44">
+        <v>4874</v>
+      </c>
+      <c r="I46" s="44">
+        <v>4871</v>
+      </c>
+      <c r="J46" s="44">
+        <v>4876</v>
+      </c>
+      <c r="K46" s="44">
+        <v>4</v>
+      </c>
+      <c r="L46" s="44">
+        <v>7</v>
+      </c>
+      <c r="M46" s="44">
+        <v>2</v>
+      </c>
       <c r="N46" s="45"/>
-      <c r="O46" s="45"/>
-      <c r="P46" s="45"/>
-      <c r="Q46" s="45"/>
-      <c r="R46" s="46" t="e">
+      <c r="O46" s="44">
+        <v>0</v>
+      </c>
+      <c r="P46" s="44">
+        <v>0</v>
+      </c>
+      <c r="Q46" s="44">
+        <v>0</v>
+      </c>
+      <c r="R46" s="46">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:18" x14ac:dyDescent="0.3">
@@ -3022,24 +3156,50 @@
       <c r="B47" s="47" t="s">
         <v>17</v>
       </c>
-      <c r="C47" s="45"/>
-      <c r="D47" s="45"/>
-      <c r="E47" s="45"/>
-      <c r="F47" s="45"/>
+      <c r="C47" s="48">
+        <v>0.99965833000000004</v>
+      </c>
+      <c r="D47" s="48">
+        <v>2.3671599999999999E-4</v>
+      </c>
+      <c r="E47" s="48">
+        <v>0.99965761399999997</v>
+      </c>
+      <c r="F47" s="48">
+        <v>2.3729999999999999E-4</v>
+      </c>
       <c r="G47" s="45"/>
-      <c r="H47" s="45"/>
-      <c r="I47" s="45"/>
-      <c r="J47" s="45"/>
-      <c r="K47" s="45"/>
-      <c r="L47" s="45"/>
-      <c r="M47" s="45"/>
+      <c r="H47" s="44">
+        <v>4877</v>
+      </c>
+      <c r="I47" s="44">
+        <v>4875</v>
+      </c>
+      <c r="J47" s="44">
+        <v>4877</v>
+      </c>
+      <c r="K47" s="44">
+        <v>1</v>
+      </c>
+      <c r="L47" s="44">
+        <v>3</v>
+      </c>
+      <c r="M47" s="44">
+        <v>1</v>
+      </c>
       <c r="N47" s="45"/>
-      <c r="O47" s="45"/>
-      <c r="P47" s="45"/>
-      <c r="Q47" s="45"/>
-      <c r="R47" s="46" t="e">
+      <c r="O47" s="44">
+        <v>0</v>
+      </c>
+      <c r="P47" s="44">
+        <v>0</v>
+      </c>
+      <c r="Q47" s="44">
+        <v>0</v>
+      </c>
+      <c r="R47" s="46">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48" spans="1:18" x14ac:dyDescent="0.3">
@@ -3049,24 +3209,50 @@
       <c r="B48" s="47" t="s">
         <v>16</v>
       </c>
-      <c r="C48" s="45"/>
-      <c r="D48" s="45"/>
-      <c r="E48" s="45"/>
-      <c r="F48" s="45"/>
+      <c r="C48" s="48">
+        <v>1</v>
+      </c>
+      <c r="D48" s="48">
+        <v>0</v>
+      </c>
+      <c r="E48" s="48">
+        <v>1</v>
+      </c>
+      <c r="F48" s="48">
+        <v>0</v>
+      </c>
       <c r="G48" s="45"/>
-      <c r="H48" s="45"/>
-      <c r="I48" s="45"/>
-      <c r="J48" s="45"/>
-      <c r="K48" s="45"/>
-      <c r="L48" s="45"/>
-      <c r="M48" s="45"/>
+      <c r="H48" s="44">
+        <v>4878</v>
+      </c>
+      <c r="I48" s="44">
+        <v>4878</v>
+      </c>
+      <c r="J48" s="44">
+        <v>4878</v>
+      </c>
+      <c r="K48" s="44">
+        <v>0</v>
+      </c>
+      <c r="L48" s="44">
+        <v>0</v>
+      </c>
+      <c r="M48" s="44">
+        <v>0</v>
+      </c>
       <c r="N48" s="45"/>
-      <c r="O48" s="45"/>
-      <c r="P48" s="45"/>
-      <c r="Q48" s="45"/>
-      <c r="R48" s="46" t="e">
+      <c r="O48" s="44">
+        <v>0</v>
+      </c>
+      <c r="P48" s="44">
+        <v>0</v>
+      </c>
+      <c r="Q48" s="44">
+        <v>0</v>
+      </c>
+      <c r="R48" s="46">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49" spans="1:18" x14ac:dyDescent="0.3">
@@ -3076,24 +3262,50 @@
       <c r="B49" s="44" t="s">
         <v>24</v>
       </c>
-      <c r="C49" s="45"/>
-      <c r="D49" s="45"/>
-      <c r="E49" s="45"/>
-      <c r="F49" s="45"/>
+      <c r="C49" s="48">
+        <v>1</v>
+      </c>
+      <c r="D49" s="48">
+        <v>0</v>
+      </c>
+      <c r="E49" s="48">
+        <v>1</v>
+      </c>
+      <c r="F49" s="48">
+        <v>0</v>
+      </c>
       <c r="G49" s="45"/>
-      <c r="H49" s="45"/>
-      <c r="I49" s="45"/>
-      <c r="J49" s="45"/>
-      <c r="K49" s="45"/>
-      <c r="L49" s="45"/>
-      <c r="M49" s="45"/>
+      <c r="H49" s="44">
+        <v>100</v>
+      </c>
+      <c r="I49" s="44">
+        <v>100</v>
+      </c>
+      <c r="J49" s="44">
+        <v>100</v>
+      </c>
+      <c r="K49" s="44">
+        <v>0</v>
+      </c>
+      <c r="L49" s="44">
+        <v>0</v>
+      </c>
+      <c r="M49" s="44">
+        <v>0</v>
+      </c>
       <c r="N49" s="45"/>
-      <c r="O49" s="45"/>
-      <c r="P49" s="45"/>
-      <c r="Q49" s="45"/>
-      <c r="R49" s="46" t="e">
+      <c r="O49" s="44">
+        <v>0</v>
+      </c>
+      <c r="P49" s="44">
+        <v>0</v>
+      </c>
+      <c r="Q49" s="44">
+        <v>0</v>
+      </c>
+      <c r="R49" s="46">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:18" x14ac:dyDescent="0.3">
@@ -3103,24 +3315,50 @@
       <c r="B50" s="44" t="s">
         <v>23</v>
       </c>
-      <c r="C50" s="45"/>
-      <c r="D50" s="45"/>
-      <c r="E50" s="45"/>
-      <c r="F50" s="45"/>
+      <c r="C50" s="48">
+        <v>1</v>
+      </c>
+      <c r="D50" s="48">
+        <v>0</v>
+      </c>
+      <c r="E50" s="48">
+        <v>1</v>
+      </c>
+      <c r="F50" s="48">
+        <v>0</v>
+      </c>
       <c r="G50" s="45"/>
-      <c r="H50" s="45"/>
-      <c r="I50" s="45"/>
-      <c r="J50" s="45"/>
-      <c r="K50" s="45"/>
-      <c r="L50" s="45"/>
-      <c r="M50" s="45"/>
+      <c r="H50" s="44">
+        <v>100</v>
+      </c>
+      <c r="I50" s="44">
+        <v>100</v>
+      </c>
+      <c r="J50" s="44">
+        <v>100</v>
+      </c>
+      <c r="K50" s="44">
+        <v>0</v>
+      </c>
+      <c r="L50" s="44">
+        <v>0</v>
+      </c>
+      <c r="M50" s="44">
+        <v>0</v>
+      </c>
       <c r="N50" s="45"/>
-      <c r="O50" s="45"/>
-      <c r="P50" s="45"/>
-      <c r="Q50" s="45"/>
-      <c r="R50" s="46" t="e">
+      <c r="O50" s="44">
+        <v>0</v>
+      </c>
+      <c r="P50" s="44">
+        <v>0</v>
+      </c>
+      <c r="Q50" s="44">
+        <v>0</v>
+      </c>
+      <c r="R50" s="46">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51" spans="1:18" x14ac:dyDescent="0.3">
@@ -3130,24 +3368,50 @@
       <c r="B51" s="44" t="s">
         <v>22</v>
       </c>
-      <c r="C51" s="45"/>
-      <c r="D51" s="45"/>
-      <c r="E51" s="45"/>
-      <c r="F51" s="45"/>
+      <c r="C51" s="48">
+        <v>1</v>
+      </c>
+      <c r="D51" s="48">
+        <v>0</v>
+      </c>
+      <c r="E51" s="48">
+        <v>1</v>
+      </c>
+      <c r="F51" s="48">
+        <v>0</v>
+      </c>
       <c r="G51" s="45"/>
-      <c r="H51" s="45"/>
-      <c r="I51" s="45"/>
-      <c r="J51" s="45"/>
-      <c r="K51" s="45"/>
-      <c r="L51" s="45"/>
-      <c r="M51" s="45"/>
+      <c r="H51" s="44">
+        <v>100</v>
+      </c>
+      <c r="I51" s="44">
+        <v>100</v>
+      </c>
+      <c r="J51" s="44">
+        <v>100</v>
+      </c>
+      <c r="K51" s="44">
+        <v>0</v>
+      </c>
+      <c r="L51" s="44">
+        <v>0</v>
+      </c>
+      <c r="M51" s="44">
+        <v>0</v>
+      </c>
       <c r="N51" s="45"/>
-      <c r="O51" s="45"/>
-      <c r="P51" s="45"/>
-      <c r="Q51" s="45"/>
-      <c r="R51" s="46" t="e">
+      <c r="O51" s="44">
+        <v>0</v>
+      </c>
+      <c r="P51" s="44">
+        <v>0</v>
+      </c>
+      <c r="Q51" s="44">
+        <v>0</v>
+      </c>
+      <c r="R51" s="46">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52" spans="1:18" x14ac:dyDescent="0.3">

</xml_diff>